<commit_message>
preserve quotation export template footer notes and bank info
</commit_message>
<xml_diff>
--- a/app/assets/quote_template.xlsx
+++ b/app/assets/quote_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevinkao/Documents/software building/b2b-quotation-system-backend/app/assets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevinkao/Documents/software building/b2b-quotation-project/b2b-quotation-system-backend/app/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6476E619-594C-3741-B04B-54A437126ACA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB5E682C-F37F-0D40-87EF-2014CDD72CA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1580" yWindow="760" windowWidth="27240" windowHeight="18360" xr2:uid="{3E340372-419D-D74C-8630-F9BDE50D3BA2}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="27040" windowHeight="16940" xr2:uid="{3E340372-419D-D74C-8630-F9BDE50D3BA2}"/>
   </bookViews>
   <sheets>
     <sheet name="1014 智慧校園 (網達)" sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t>Address  臺北市信義區基隆路一段206號18樓   /   Tel  02 7709 7001  /  Cellphone  0988 697 165  /   Tax Number  82817282</t>
   </si>
@@ -113,33 +113,6 @@
   </si>
   <si>
     <t>小計</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>進場安裝搭建執行及撤場清運</t>
-  </si>
-  <si>
-    <t>製作施工</t>
-  </si>
-  <si>
-    <t>尺寸：250*400*30cm</t>
-  </si>
-  <si>
-    <t>Partation 結構（黑）</t>
-  </si>
-  <si>
-    <t>展場結構</t>
-  </si>
-  <si>
-    <t>展位牆面圖面輸出</t>
-  </si>
-  <si>
-    <t>展場輸出</t>
   </si>
   <si>
     <r>
@@ -178,18 +151,6 @@
   </si>
   <si>
     <t>項次</t>
-  </si>
-  <si>
-    <t>台北六福萬怡 7樓 超新星廳</t>
-  </si>
-  <si>
-    <t>地點</t>
-  </si>
-  <si>
-    <t>01/28 15:00 進場 21:00 撤場</t>
-  </si>
-  <si>
-    <t>展期</t>
   </si>
   <si>
     <t>項目名稱</t>
@@ -632,10 +593,106 @@
     <xf numFmtId="41" fontId="20" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="21" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="41" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="180" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="41" fontId="20" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -644,104 +701,8 @@
     <xf numFmtId="41" fontId="20" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="20" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="21" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="41" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1244,10 +1205,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:18">
-      <c r="L1" s="84" t="s">
-        <v>55</v>
-      </c>
-      <c r="M1" s="84"/>
+      <c r="L1" s="60" t="s">
+        <v>42</v>
+      </c>
+      <c r="M1" s="60"/>
     </row>
     <row r="2" spans="2:18" ht="21" customHeight="1">
       <c r="B2" s="13"/>
@@ -1256,13 +1217,13 @@
       <c r="E2" s="13"/>
       <c r="F2" s="5"/>
       <c r="G2" s="13"/>
-      <c r="H2" s="85" t="s">
-        <v>54</v>
-      </c>
-      <c r="I2" s="86"/>
-      <c r="J2" s="86"/>
-      <c r="K2" s="86"/>
-      <c r="L2" s="86"/>
+      <c r="H2" s="61" t="s">
+        <v>41</v>
+      </c>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="62"/>
+      <c r="L2" s="62"/>
     </row>
     <row r="3" spans="2:18" ht="21" customHeight="1">
       <c r="B3" s="13"/>
@@ -1271,11 +1232,11 @@
       <c r="E3" s="13"/>
       <c r="F3" s="5"/>
       <c r="G3" s="13"/>
-      <c r="H3" s="86"/>
-      <c r="I3" s="86"/>
-      <c r="J3" s="86"/>
-      <c r="K3" s="86"/>
-      <c r="L3" s="86"/>
+      <c r="H3" s="62"/>
+      <c r="I3" s="62"/>
+      <c r="J3" s="62"/>
+      <c r="K3" s="62"/>
+      <c r="L3" s="62"/>
     </row>
     <row r="4" spans="2:18" ht="34" customHeight="1">
       <c r="B4" s="13"/>
@@ -1289,141 +1250,133 @@
       <c r="J4" s="5"/>
     </row>
     <row r="5" spans="2:18" ht="21">
-      <c r="B5" s="71"/>
-      <c r="C5" s="71"/>
-      <c r="D5" s="71"/>
-      <c r="E5" s="71"/>
+      <c r="B5" s="56"/>
+      <c r="C5" s="56"/>
+      <c r="D5" s="56"/>
+      <c r="E5" s="56"/>
       <c r="F5" s="5"/>
       <c r="I5" s="48" t="s">
-        <v>53</v>
-      </c>
-      <c r="J5" s="80" t="s">
-        <v>52</v>
-      </c>
-      <c r="K5" s="80"/>
-      <c r="L5" s="80"/>
+        <v>40</v>
+      </c>
+      <c r="J5" s="53" t="s">
+        <v>39</v>
+      </c>
+      <c r="K5" s="53"/>
+      <c r="L5" s="53"/>
     </row>
     <row r="6" spans="2:18" ht="26" customHeight="1">
-      <c r="B6" s="71"/>
-      <c r="C6" s="71"/>
-      <c r="D6" s="71"/>
-      <c r="E6" s="71"/>
+      <c r="B6" s="56"/>
+      <c r="C6" s="56"/>
+      <c r="D6" s="56"/>
+      <c r="E6" s="56"/>
       <c r="F6" s="5"/>
       <c r="I6" s="48" t="s">
-        <v>51</v>
-      </c>
-      <c r="J6" s="80" t="s">
-        <v>50</v>
-      </c>
-      <c r="K6" s="80"/>
-      <c r="L6" s="80"/>
+        <v>38</v>
+      </c>
+      <c r="J6" s="53" t="s">
+        <v>37</v>
+      </c>
+      <c r="K6" s="53"/>
+      <c r="L6" s="53"/>
     </row>
     <row r="7" spans="2:18" ht="26" customHeight="1">
-      <c r="B7" s="71"/>
-      <c r="C7" s="71"/>
-      <c r="D7" s="71"/>
-      <c r="E7" s="71"/>
+      <c r="B7" s="56"/>
+      <c r="C7" s="56"/>
+      <c r="D7" s="56"/>
+      <c r="E7" s="56"/>
       <c r="F7" s="5"/>
       <c r="I7" s="48" t="s">
-        <v>49</v>
-      </c>
-      <c r="J7" s="80" t="s">
-        <v>48</v>
-      </c>
-      <c r="K7" s="80"/>
-      <c r="L7" s="80"/>
+        <v>36</v>
+      </c>
+      <c r="J7" s="53" t="s">
+        <v>35</v>
+      </c>
+      <c r="K7" s="53"/>
+      <c r="L7" s="53"/>
     </row>
     <row r="8" spans="2:18" ht="26" customHeight="1">
-      <c r="B8" s="71"/>
-      <c r="C8" s="71"/>
-      <c r="D8" s="71"/>
-      <c r="E8" s="71"/>
+      <c r="B8" s="56"/>
+      <c r="C8" s="56"/>
+      <c r="D8" s="56"/>
+      <c r="E8" s="56"/>
       <c r="F8" s="5"/>
       <c r="H8" s="8"/>
       <c r="I8" s="48" t="s">
-        <v>47</v>
-      </c>
-      <c r="J8" s="80" t="s">
-        <v>46</v>
-      </c>
-      <c r="K8" s="80"/>
-      <c r="L8" s="80"/>
+        <v>34</v>
+      </c>
+      <c r="J8" s="53" t="s">
+        <v>33</v>
+      </c>
+      <c r="K8" s="53"/>
+      <c r="L8" s="53"/>
     </row>
     <row r="9" spans="2:18" ht="21">
-      <c r="B9" s="71"/>
-      <c r="C9" s="71"/>
-      <c r="D9" s="71"/>
-      <c r="E9" s="71"/>
+      <c r="B9" s="56"/>
+      <c r="C9" s="56"/>
+      <c r="D9" s="56"/>
+      <c r="E9" s="56"/>
       <c r="F9" s="5"/>
       <c r="I9" s="48" t="s">
-        <v>45</v>
-      </c>
-      <c r="J9" s="80" t="s">
-        <v>44</v>
-      </c>
-      <c r="K9" s="80"/>
-      <c r="L9" s="80"/>
+        <v>32</v>
+      </c>
+      <c r="J9" s="53" t="s">
+        <v>31</v>
+      </c>
+      <c r="K9" s="53"/>
+      <c r="L9" s="53"/>
     </row>
     <row r="10" spans="2:18" ht="28" customHeight="1">
-      <c r="B10" s="71"/>
-      <c r="C10" s="71"/>
-      <c r="D10" s="71"/>
-      <c r="E10" s="71"/>
+      <c r="B10" s="56"/>
+      <c r="C10" s="56"/>
+      <c r="D10" s="56"/>
+      <c r="E10" s="56"/>
       <c r="F10" s="5"/>
       <c r="I10" s="48" t="s">
-        <v>43</v>
-      </c>
-      <c r="J10" s="87"/>
-      <c r="K10" s="87"/>
-      <c r="L10" s="87"/>
+        <v>30</v>
+      </c>
+      <c r="J10" s="63"/>
+      <c r="K10" s="63"/>
+      <c r="L10" s="63"/>
     </row>
     <row r="11" spans="2:18" ht="21" customHeight="1">
-      <c r="B11" s="71"/>
-      <c r="C11" s="71"/>
-      <c r="D11" s="71"/>
-      <c r="E11" s="71"/>
+      <c r="B11" s="56"/>
+      <c r="C11" s="56"/>
+      <c r="D11" s="56"/>
+      <c r="E11" s="56"/>
       <c r="F11" s="5"/>
       <c r="G11" s="13"/>
       <c r="H11" s="8"/>
       <c r="I11" s="13"/>
-      <c r="J11" s="87"/>
-      <c r="K11" s="87"/>
-      <c r="L11" s="87"/>
+      <c r="J11" s="63"/>
+      <c r="K11" s="63"/>
+      <c r="L11" s="63"/>
     </row>
     <row r="12" spans="2:18" ht="21" customHeight="1">
-      <c r="B12" s="71"/>
-      <c r="C12" s="71"/>
-      <c r="D12" s="71"/>
-      <c r="E12" s="71"/>
-      <c r="J12" s="87"/>
-      <c r="K12" s="87"/>
-      <c r="L12" s="87"/>
+      <c r="B12" s="56"/>
+      <c r="C12" s="56"/>
+      <c r="D12" s="56"/>
+      <c r="E12" s="56"/>
+      <c r="J12" s="63"/>
+      <c r="K12" s="63"/>
+      <c r="L12" s="63"/>
     </row>
     <row r="13" spans="2:18" ht="21">
       <c r="B13" s="13"/>
       <c r="C13" s="13"/>
       <c r="D13" s="13"/>
-      <c r="I13" s="48" t="s">
-        <v>42</v>
-      </c>
-      <c r="J13" s="78" t="s">
-        <v>41</v>
-      </c>
-      <c r="K13" s="79"/>
-      <c r="L13" s="79"/>
+      <c r="I13" s="48"/>
+      <c r="J13" s="51"/>
+      <c r="K13" s="52"/>
+      <c r="L13" s="52"/>
     </row>
     <row r="14" spans="2:18" ht="21" customHeight="1">
       <c r="B14" s="13"/>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
-      <c r="I14" s="48" t="s">
-        <v>40</v>
-      </c>
-      <c r="J14" s="80" t="s">
-        <v>39</v>
-      </c>
-      <c r="K14" s="80"/>
-      <c r="L14" s="80"/>
+      <c r="I14" s="48"/>
+      <c r="J14" s="53"/>
+      <c r="K14" s="53"/>
+      <c r="L14" s="53"/>
     </row>
     <row r="15" spans="2:18" ht="21" customHeight="1">
       <c r="B15" s="13"/>
@@ -1439,24 +1392,24 @@
       <c r="C16" s="13"/>
       <c r="D16" s="13"/>
       <c r="E16" s="46" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="F16" s="45" t="s">
-        <v>37</v>
-      </c>
-      <c r="G16" s="81" t="s">
-        <v>36</v>
-      </c>
-      <c r="H16" s="81"/>
-      <c r="I16" s="81"/>
+        <v>28</v>
+      </c>
+      <c r="G16" s="54" t="s">
+        <v>27</v>
+      </c>
+      <c r="H16" s="54"/>
+      <c r="I16" s="54"/>
       <c r="J16" s="45" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="K16" s="44" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="L16" s="44" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="O16" s="1"/>
       <c r="Q16" s="1"/>
@@ -1466,26 +1419,18 @@
       <c r="B17" s="13"/>
       <c r="C17" s="13"/>
       <c r="D17" s="13"/>
-      <c r="E17" s="82">
+      <c r="E17" s="55">
         <v>1</v>
       </c>
-      <c r="F17" s="83" t="s">
-        <v>32</v>
-      </c>
-      <c r="G17" s="67" t="s">
-        <v>31</v>
-      </c>
-      <c r="H17" s="67"/>
-      <c r="I17" s="67"/>
-      <c r="J17" s="64" t="s">
-        <v>25</v>
-      </c>
-      <c r="K17" s="53">
-        <v>35000</v>
-      </c>
-      <c r="L17" s="53">
+      <c r="F17" s="57"/>
+      <c r="G17" s="59"/>
+      <c r="H17" s="59"/>
+      <c r="I17" s="59"/>
+      <c r="J17" s="87"/>
+      <c r="K17" s="85"/>
+      <c r="L17" s="85">
         <f>J17*K17</f>
-        <v>35000</v>
+        <v>0</v>
       </c>
       <c r="Q17" s="42"/>
     </row>
@@ -1493,36 +1438,28 @@
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
-      <c r="E18" s="71"/>
-      <c r="F18" s="52"/>
-      <c r="G18" s="61" t="s">
-        <v>28</v>
-      </c>
-      <c r="H18" s="61"/>
-      <c r="I18" s="61"/>
-      <c r="J18" s="63"/>
-      <c r="K18" s="54"/>
-      <c r="L18" s="54"/>
+      <c r="E18" s="56"/>
+      <c r="F18" s="58"/>
+      <c r="G18" s="68"/>
+      <c r="H18" s="68"/>
+      <c r="I18" s="68"/>
+      <c r="J18" s="65"/>
+      <c r="K18" s="86"/>
+      <c r="L18" s="86"/>
       <c r="O18" s="43"/>
     </row>
     <row r="19" spans="2:19" ht="21" customHeight="1">
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
       <c r="D19" s="13"/>
-      <c r="E19" s="68">
+      <c r="E19" s="69">
         <v>2</v>
       </c>
-      <c r="F19" s="51" t="s">
-        <v>30</v>
-      </c>
-      <c r="G19" s="67" t="s">
-        <v>29</v>
-      </c>
-      <c r="H19" s="67"/>
-      <c r="I19" s="67"/>
-      <c r="J19" s="62" t="s">
-        <v>25</v>
-      </c>
+      <c r="F19" s="71"/>
+      <c r="G19" s="59"/>
+      <c r="H19" s="59"/>
+      <c r="I19" s="59"/>
+      <c r="J19" s="64"/>
       <c r="K19" s="49"/>
       <c r="L19" s="49"/>
       <c r="Q19" s="42"/>
@@ -1531,14 +1468,12 @@
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
-      <c r="E20" s="69"/>
-      <c r="F20" s="52"/>
-      <c r="G20" s="61" t="s">
-        <v>28</v>
-      </c>
-      <c r="H20" s="61"/>
-      <c r="I20" s="61"/>
-      <c r="J20" s="63"/>
+      <c r="E20" s="70"/>
+      <c r="F20" s="58"/>
+      <c r="G20" s="68"/>
+      <c r="H20" s="68"/>
+      <c r="I20" s="68"/>
+      <c r="J20" s="65"/>
       <c r="K20" s="49"/>
       <c r="L20" s="49"/>
     </row>
@@ -1546,20 +1481,14 @@
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
-      <c r="E21" s="68">
+      <c r="E21" s="69">
         <v>2</v>
       </c>
-      <c r="F21" s="51" t="s">
-        <v>27</v>
-      </c>
-      <c r="G21" s="67" t="s">
-        <v>26</v>
-      </c>
-      <c r="H21" s="67"/>
-      <c r="I21" s="67"/>
-      <c r="J21" s="62" t="s">
-        <v>25</v>
-      </c>
+      <c r="F21" s="71"/>
+      <c r="G21" s="59"/>
+      <c r="H21" s="59"/>
+      <c r="I21" s="59"/>
+      <c r="J21" s="64"/>
       <c r="K21" s="49"/>
       <c r="L21" s="49"/>
       <c r="Q21" s="42"/>
@@ -1568,342 +1497,340 @@
       <c r="B22" s="13"/>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
-      <c r="E22" s="69"/>
-      <c r="F22" s="52"/>
-      <c r="G22" s="61"/>
-      <c r="H22" s="61"/>
-      <c r="I22" s="61"/>
-      <c r="J22" s="63"/>
+      <c r="E22" s="70"/>
+      <c r="F22" s="58"/>
+      <c r="G22" s="68"/>
+      <c r="H22" s="68"/>
+      <c r="I22" s="68"/>
+      <c r="J22" s="65"/>
       <c r="K22" s="50"/>
       <c r="L22" s="50"/>
       <c r="P22"/>
     </row>
     <row r="23" spans="2:19" ht="21" customHeight="1">
-      <c r="E23" s="71"/>
-      <c r="F23" s="51"/>
-      <c r="G23" s="67"/>
-      <c r="H23" s="67"/>
-      <c r="I23" s="67"/>
-      <c r="J23" s="62"/>
-      <c r="K23" s="65"/>
-      <c r="L23" s="65"/>
+      <c r="E23" s="56"/>
+      <c r="F23" s="71"/>
+      <c r="G23" s="59"/>
+      <c r="H23" s="59"/>
+      <c r="I23" s="59"/>
+      <c r="J23" s="64"/>
+      <c r="K23" s="66"/>
+      <c r="L23" s="66"/>
       <c r="Q23" s="18"/>
       <c r="S23" s="8"/>
     </row>
     <row r="24" spans="2:19" ht="21" customHeight="1">
-      <c r="E24" s="69"/>
-      <c r="F24" s="52"/>
-      <c r="G24" s="61"/>
-      <c r="H24" s="61"/>
-      <c r="I24" s="61"/>
-      <c r="J24" s="63"/>
-      <c r="K24" s="66"/>
-      <c r="L24" s="66"/>
+      <c r="E24" s="70"/>
+      <c r="F24" s="58"/>
+      <c r="G24" s="68"/>
+      <c r="H24" s="68"/>
+      <c r="I24" s="68"/>
+      <c r="J24" s="65"/>
+      <c r="K24" s="67"/>
+      <c r="L24" s="67"/>
       <c r="S24" s="8"/>
     </row>
     <row r="25" spans="2:19" ht="21" customHeight="1">
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
       <c r="D25" s="13"/>
-      <c r="E25" s="71"/>
-      <c r="F25" s="51"/>
-      <c r="G25" s="67"/>
-      <c r="H25" s="67"/>
-      <c r="I25" s="67"/>
-      <c r="J25" s="62"/>
-      <c r="K25" s="65"/>
-      <c r="L25" s="65"/>
+      <c r="E25" s="56"/>
+      <c r="F25" s="71"/>
+      <c r="G25" s="59"/>
+      <c r="H25" s="59"/>
+      <c r="I25" s="59"/>
+      <c r="J25" s="64"/>
+      <c r="K25" s="66"/>
+      <c r="L25" s="66"/>
       <c r="Q25" s="42"/>
     </row>
     <row r="26" spans="2:19" ht="21" customHeight="1">
       <c r="B26" s="13"/>
       <c r="C26" s="13"/>
       <c r="D26" s="13"/>
-      <c r="E26" s="69"/>
-      <c r="F26" s="52"/>
-      <c r="G26" s="61"/>
-      <c r="H26" s="61"/>
-      <c r="I26" s="61"/>
-      <c r="J26" s="63"/>
-      <c r="K26" s="66"/>
-      <c r="L26" s="66"/>
+      <c r="E26" s="70"/>
+      <c r="F26" s="58"/>
+      <c r="G26" s="68"/>
+      <c r="H26" s="68"/>
+      <c r="I26" s="68"/>
+      <c r="J26" s="65"/>
+      <c r="K26" s="67"/>
+      <c r="L26" s="67"/>
     </row>
     <row r="27" spans="2:19" ht="21" customHeight="1">
       <c r="B27" s="13"/>
       <c r="C27" s="13"/>
       <c r="D27" s="13"/>
-      <c r="E27" s="71"/>
-      <c r="F27" s="51"/>
-      <c r="G27" s="67"/>
-      <c r="H27" s="67"/>
-      <c r="I27" s="67"/>
-      <c r="J27" s="62"/>
-      <c r="K27" s="65"/>
-      <c r="L27" s="65"/>
+      <c r="E27" s="56"/>
+      <c r="F27" s="71"/>
+      <c r="G27" s="59"/>
+      <c r="H27" s="59"/>
+      <c r="I27" s="59"/>
+      <c r="J27" s="64"/>
+      <c r="K27" s="66"/>
+      <c r="L27" s="66"/>
       <c r="Q27" s="42"/>
     </row>
     <row r="28" spans="2:19" ht="21" customHeight="1">
       <c r="B28" s="13"/>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
-      <c r="E28" s="69"/>
-      <c r="F28" s="52"/>
-      <c r="G28" s="61"/>
-      <c r="H28" s="61"/>
-      <c r="I28" s="61"/>
-      <c r="J28" s="63"/>
-      <c r="K28" s="66"/>
-      <c r="L28" s="66"/>
+      <c r="E28" s="70"/>
+      <c r="F28" s="58"/>
+      <c r="G28" s="68"/>
+      <c r="H28" s="68"/>
+      <c r="I28" s="68"/>
+      <c r="J28" s="65"/>
+      <c r="K28" s="67"/>
+      <c r="L28" s="67"/>
     </row>
     <row r="29" spans="2:19" ht="21" customHeight="1">
-      <c r="E29" s="71"/>
-      <c r="F29" s="51"/>
-      <c r="G29" s="67"/>
-      <c r="H29" s="67"/>
-      <c r="I29" s="67"/>
-      <c r="J29" s="62"/>
-      <c r="K29" s="65"/>
-      <c r="L29" s="65"/>
+      <c r="E29" s="56"/>
+      <c r="F29" s="71"/>
+      <c r="G29" s="59"/>
+      <c r="H29" s="59"/>
+      <c r="I29" s="59"/>
+      <c r="J29" s="64"/>
+      <c r="K29" s="66"/>
+      <c r="L29" s="66"/>
       <c r="Q29" s="18"/>
       <c r="S29" s="8"/>
     </row>
     <row r="30" spans="2:19" ht="21" customHeight="1">
-      <c r="E30" s="69"/>
-      <c r="F30" s="52"/>
-      <c r="G30" s="61"/>
-      <c r="H30" s="61"/>
-      <c r="I30" s="61"/>
-      <c r="J30" s="63"/>
-      <c r="K30" s="66"/>
-      <c r="L30" s="66"/>
+      <c r="E30" s="70"/>
+      <c r="F30" s="58"/>
+      <c r="G30" s="68"/>
+      <c r="H30" s="68"/>
+      <c r="I30" s="68"/>
+      <c r="J30" s="65"/>
+      <c r="K30" s="67"/>
+      <c r="L30" s="67"/>
       <c r="S30" s="8"/>
     </row>
     <row r="31" spans="2:19" ht="21" customHeight="1">
-      <c r="E31" s="71"/>
-      <c r="F31" s="51"/>
-      <c r="G31" s="67"/>
-      <c r="H31" s="67"/>
-      <c r="I31" s="67"/>
-      <c r="J31" s="62"/>
-      <c r="K31" s="65"/>
-      <c r="L31" s="65"/>
+      <c r="E31" s="56"/>
+      <c r="F31" s="71"/>
+      <c r="G31" s="59"/>
+      <c r="H31" s="59"/>
+      <c r="I31" s="59"/>
+      <c r="J31" s="64"/>
+      <c r="K31" s="66"/>
+      <c r="L31" s="66"/>
       <c r="Q31" s="18"/>
       <c r="S31" s="8"/>
     </row>
     <row r="32" spans="2:19" ht="21" customHeight="1">
-      <c r="E32" s="69"/>
-      <c r="F32" s="52"/>
-      <c r="G32" s="61"/>
-      <c r="H32" s="61"/>
-      <c r="I32" s="61"/>
-      <c r="J32" s="63"/>
-      <c r="K32" s="66"/>
-      <c r="L32" s="66"/>
+      <c r="E32" s="70"/>
+      <c r="F32" s="58"/>
+      <c r="G32" s="68"/>
+      <c r="H32" s="68"/>
+      <c r="I32" s="68"/>
+      <c r="J32" s="65"/>
+      <c r="K32" s="67"/>
+      <c r="L32" s="67"/>
       <c r="S32" s="8"/>
     </row>
     <row r="33" spans="2:19" ht="21" customHeight="1">
-      <c r="E33" s="71"/>
-      <c r="F33" s="51"/>
-      <c r="G33" s="67"/>
-      <c r="H33" s="67"/>
-      <c r="I33" s="67"/>
-      <c r="J33" s="62"/>
-      <c r="K33" s="76"/>
-      <c r="L33" s="76"/>
+      <c r="E33" s="56"/>
+      <c r="F33" s="71"/>
+      <c r="G33" s="59"/>
+      <c r="H33" s="59"/>
+      <c r="I33" s="59"/>
+      <c r="J33" s="64"/>
+      <c r="K33" s="72"/>
+      <c r="L33" s="72"/>
       <c r="Q33" s="18"/>
       <c r="S33" s="8"/>
     </row>
     <row r="34" spans="2:19" ht="21" customHeight="1">
-      <c r="E34" s="71"/>
-      <c r="F34" s="51"/>
-      <c r="G34" s="77" t="s">
-        <v>24</v>
-      </c>
-      <c r="H34" s="77"/>
-      <c r="I34" s="77"/>
-      <c r="J34" s="62"/>
-      <c r="K34" s="76"/>
-      <c r="L34" s="76"/>
+      <c r="E34" s="56"/>
+      <c r="F34" s="71"/>
+      <c r="G34" s="73"/>
+      <c r="H34" s="73"/>
+      <c r="I34" s="73"/>
+      <c r="J34" s="64"/>
+      <c r="K34" s="72"/>
+      <c r="L34" s="72"/>
       <c r="S34" s="8"/>
     </row>
     <row r="35" spans="2:19" ht="21" customHeight="1">
       <c r="B35" s="13"/>
       <c r="C35" s="13"/>
       <c r="D35" s="13"/>
-      <c r="E35" s="71"/>
-      <c r="F35" s="51"/>
-      <c r="G35" s="67"/>
-      <c r="H35" s="67"/>
-      <c r="I35" s="67"/>
-      <c r="J35" s="62"/>
-      <c r="K35" s="76"/>
-      <c r="L35" s="76"/>
+      <c r="E35" s="56"/>
+      <c r="F35" s="71"/>
+      <c r="G35" s="59"/>
+      <c r="H35" s="59"/>
+      <c r="I35" s="59"/>
+      <c r="J35" s="64"/>
+      <c r="K35" s="72"/>
+      <c r="L35" s="72"/>
       <c r="Q35" s="42"/>
     </row>
     <row r="36" spans="2:19" ht="23" customHeight="1">
       <c r="B36" s="13"/>
       <c r="C36" s="13"/>
       <c r="D36" s="13"/>
-      <c r="E36" s="71"/>
-      <c r="F36" s="51"/>
-      <c r="G36" s="77"/>
-      <c r="H36" s="77"/>
-      <c r="I36" s="77"/>
-      <c r="J36" s="62"/>
-      <c r="K36" s="76"/>
-      <c r="L36" s="76"/>
+      <c r="E36" s="56"/>
+      <c r="F36" s="71"/>
+      <c r="G36" s="73"/>
+      <c r="H36" s="73"/>
+      <c r="I36" s="73"/>
+      <c r="J36" s="64"/>
+      <c r="K36" s="72"/>
+      <c r="L36" s="72"/>
     </row>
     <row r="37" spans="2:19" ht="21" customHeight="1">
-      <c r="E37" s="71"/>
-      <c r="F37" s="51"/>
-      <c r="G37" s="67"/>
-      <c r="H37" s="67"/>
-      <c r="I37" s="67"/>
-      <c r="J37" s="62"/>
-      <c r="K37" s="76"/>
-      <c r="L37" s="76"/>
+      <c r="E37" s="56"/>
+      <c r="F37" s="71"/>
+      <c r="G37" s="59"/>
+      <c r="H37" s="59"/>
+      <c r="I37" s="59"/>
+      <c r="J37" s="64"/>
+      <c r="K37" s="72"/>
+      <c r="L37" s="72"/>
       <c r="Q37" s="18"/>
       <c r="S37" s="8"/>
     </row>
     <row r="38" spans="2:19" ht="21" customHeight="1">
-      <c r="E38" s="71"/>
-      <c r="F38" s="51"/>
-      <c r="G38" s="77"/>
-      <c r="H38" s="77"/>
-      <c r="I38" s="77"/>
-      <c r="J38" s="62"/>
-      <c r="K38" s="76"/>
-      <c r="L38" s="76"/>
+      <c r="E38" s="56"/>
+      <c r="F38" s="71"/>
+      <c r="G38" s="73"/>
+      <c r="H38" s="73"/>
+      <c r="I38" s="73"/>
+      <c r="J38" s="64"/>
+      <c r="K38" s="72"/>
+      <c r="L38" s="72"/>
       <c r="S38" s="8"/>
     </row>
     <row r="39" spans="2:19" ht="21" customHeight="1">
-      <c r="E39" s="55"/>
-      <c r="F39" s="56"/>
-      <c r="G39" s="57"/>
-      <c r="H39" s="57"/>
-      <c r="I39" s="57"/>
-      <c r="J39" s="58"/>
-      <c r="K39" s="59"/>
-      <c r="L39" s="59"/>
+      <c r="E39" s="84"/>
+      <c r="F39" s="81"/>
+      <c r="G39" s="82"/>
+      <c r="H39" s="82"/>
+      <c r="I39" s="82"/>
+      <c r="J39" s="83"/>
+      <c r="K39" s="79"/>
+      <c r="L39" s="79"/>
       <c r="Q39" s="18"/>
       <c r="S39" s="8"/>
     </row>
     <row r="40" spans="2:19" ht="21" customHeight="1">
-      <c r="E40" s="55"/>
-      <c r="F40" s="56"/>
-      <c r="G40" s="60"/>
-      <c r="H40" s="60"/>
-      <c r="I40" s="60"/>
-      <c r="J40" s="58"/>
-      <c r="K40" s="59"/>
-      <c r="L40" s="59"/>
+      <c r="E40" s="84"/>
+      <c r="F40" s="81"/>
+      <c r="G40" s="80"/>
+      <c r="H40" s="80"/>
+      <c r="I40" s="80"/>
+      <c r="J40" s="83"/>
+      <c r="K40" s="79"/>
+      <c r="L40" s="79"/>
       <c r="S40" s="8"/>
     </row>
     <row r="41" spans="2:19" ht="21" customHeight="1">
-      <c r="E41" s="55"/>
-      <c r="F41" s="56"/>
-      <c r="G41" s="57"/>
-      <c r="H41" s="57"/>
-      <c r="I41" s="57"/>
-      <c r="J41" s="58"/>
-      <c r="K41" s="59"/>
-      <c r="L41" s="59"/>
+      <c r="E41" s="84"/>
+      <c r="F41" s="81"/>
+      <c r="G41" s="82"/>
+      <c r="H41" s="82"/>
+      <c r="I41" s="82"/>
+      <c r="J41" s="83"/>
+      <c r="K41" s="79"/>
+      <c r="L41" s="79"/>
       <c r="Q41" s="18"/>
       <c r="S41" s="8"/>
     </row>
     <row r="42" spans="2:19" ht="21" customHeight="1">
-      <c r="E42" s="55"/>
-      <c r="F42" s="56"/>
-      <c r="G42" s="60"/>
-      <c r="H42" s="60"/>
-      <c r="I42" s="60"/>
-      <c r="J42" s="58"/>
-      <c r="K42" s="59"/>
-      <c r="L42" s="59"/>
+      <c r="E42" s="84"/>
+      <c r="F42" s="81"/>
+      <c r="G42" s="80"/>
+      <c r="H42" s="80"/>
+      <c r="I42" s="80"/>
+      <c r="J42" s="83"/>
+      <c r="K42" s="79"/>
+      <c r="L42" s="79"/>
       <c r="S42" s="8"/>
     </row>
     <row r="43" spans="2:19" ht="21" customHeight="1">
-      <c r="E43" s="55"/>
-      <c r="F43" s="56"/>
-      <c r="G43" s="57"/>
-      <c r="H43" s="57"/>
-      <c r="I43" s="57"/>
-      <c r="J43" s="58"/>
-      <c r="K43" s="59"/>
-      <c r="L43" s="59"/>
+      <c r="E43" s="84"/>
+      <c r="F43" s="81"/>
+      <c r="G43" s="82"/>
+      <c r="H43" s="82"/>
+      <c r="I43" s="82"/>
+      <c r="J43" s="83"/>
+      <c r="K43" s="79"/>
+      <c r="L43" s="79"/>
       <c r="Q43" s="18"/>
       <c r="S43" s="8"/>
     </row>
     <row r="44" spans="2:19" ht="21" customHeight="1">
-      <c r="E44" s="55"/>
-      <c r="F44" s="56"/>
-      <c r="G44" s="60"/>
-      <c r="H44" s="60"/>
-      <c r="I44" s="60"/>
-      <c r="J44" s="58"/>
-      <c r="K44" s="59"/>
-      <c r="L44" s="59"/>
+      <c r="E44" s="84"/>
+      <c r="F44" s="81"/>
+      <c r="G44" s="80"/>
+      <c r="H44" s="80"/>
+      <c r="I44" s="80"/>
+      <c r="J44" s="83"/>
+      <c r="K44" s="79"/>
+      <c r="L44" s="79"/>
       <c r="S44" s="8"/>
     </row>
     <row r="45" spans="2:19" ht="21" customHeight="1">
-      <c r="E45" s="55"/>
-      <c r="F45" s="56"/>
-      <c r="G45" s="57"/>
-      <c r="H45" s="57"/>
-      <c r="I45" s="57"/>
-      <c r="J45" s="58"/>
-      <c r="K45" s="59"/>
-      <c r="L45" s="59"/>
+      <c r="E45" s="84"/>
+      <c r="F45" s="81"/>
+      <c r="G45" s="82"/>
+      <c r="H45" s="82"/>
+      <c r="I45" s="82"/>
+      <c r="J45" s="83"/>
+      <c r="K45" s="79"/>
+      <c r="L45" s="79"/>
       <c r="Q45" s="18"/>
       <c r="S45" s="8"/>
     </row>
     <row r="46" spans="2:19" ht="21" customHeight="1">
-      <c r="E46" s="55"/>
-      <c r="F46" s="56"/>
-      <c r="G46" s="60"/>
-      <c r="H46" s="60"/>
-      <c r="I46" s="60"/>
-      <c r="J46" s="58"/>
-      <c r="K46" s="59"/>
-      <c r="L46" s="59"/>
+      <c r="E46" s="84"/>
+      <c r="F46" s="81"/>
+      <c r="G46" s="80"/>
+      <c r="H46" s="80"/>
+      <c r="I46" s="80"/>
+      <c r="J46" s="83"/>
+      <c r="K46" s="79"/>
+      <c r="L46" s="79"/>
       <c r="S46" s="8"/>
     </row>
     <row r="47" spans="2:19" ht="21" customHeight="1">
-      <c r="E47" s="55"/>
-      <c r="F47" s="56"/>
-      <c r="G47" s="57"/>
-      <c r="H47" s="57"/>
-      <c r="I47" s="57"/>
-      <c r="J47" s="58"/>
-      <c r="K47" s="59"/>
-      <c r="L47" s="59"/>
+      <c r="E47" s="84"/>
+      <c r="F47" s="81"/>
+      <c r="G47" s="82"/>
+      <c r="H47" s="82"/>
+      <c r="I47" s="82"/>
+      <c r="J47" s="83"/>
+      <c r="K47" s="79"/>
+      <c r="L47" s="79"/>
       <c r="Q47" s="18"/>
       <c r="S47" s="8"/>
     </row>
     <row r="48" spans="2:19" ht="21" customHeight="1">
-      <c r="E48" s="55"/>
-      <c r="F48" s="56"/>
-      <c r="G48" s="60"/>
-      <c r="H48" s="60"/>
-      <c r="I48" s="60"/>
-      <c r="J48" s="58"/>
-      <c r="K48" s="59"/>
-      <c r="L48" s="59"/>
+      <c r="E48" s="84"/>
+      <c r="F48" s="81"/>
+      <c r="G48" s="80"/>
+      <c r="H48" s="80"/>
+      <c r="I48" s="80"/>
+      <c r="J48" s="83"/>
+      <c r="K48" s="79"/>
+      <c r="L48" s="79"/>
       <c r="S48" s="8"/>
     </row>
     <row r="49" spans="2:21" ht="21" customHeight="1">
-      <c r="E49" s="71"/>
-      <c r="F49" s="51"/>
-      <c r="G49" s="72"/>
-      <c r="H49" s="72"/>
-      <c r="I49" s="72"/>
+      <c r="E49" s="56"/>
+      <c r="F49" s="71"/>
+      <c r="G49" s="75"/>
+      <c r="H49" s="75"/>
+      <c r="I49" s="75"/>
       <c r="J49" s="41"/>
       <c r="K49" s="40" t="s">
         <v>23</v>
       </c>
       <c r="L49" s="39">
         <f>SUM(L17:L48)</f>
-        <v>35000</v>
+        <v>0</v>
       </c>
       <c r="N49" s="8"/>
       <c r="O49" s="8"/>
@@ -1911,18 +1838,18 @@
       <c r="S49" s="8"/>
     </row>
     <row r="50" spans="2:21" ht="21" customHeight="1">
-      <c r="E50" s="71"/>
-      <c r="F50" s="51"/>
-      <c r="G50" s="73"/>
-      <c r="H50" s="73"/>
-      <c r="I50" s="73"/>
+      <c r="E50" s="56"/>
+      <c r="F50" s="71"/>
+      <c r="G50" s="76"/>
+      <c r="H50" s="76"/>
+      <c r="I50" s="76"/>
       <c r="J50" s="38"/>
       <c r="K50" s="37" t="s">
         <v>22</v>
       </c>
       <c r="L50" s="36">
         <f>L51-L49</f>
-        <v>1750</v>
+        <v>0</v>
       </c>
       <c r="N50" s="11"/>
       <c r="O50" s="8"/>
@@ -1938,7 +1865,7 @@
       </c>
       <c r="L51" s="33">
         <f>L49*1.05</f>
-        <v>36750</v>
+        <v>0</v>
       </c>
       <c r="N51" s="11"/>
       <c r="O51" s="8"/>
@@ -1994,15 +1921,15 @@
         <v>20</v>
       </c>
       <c r="E56" s="28"/>
-      <c r="F56" s="74" t="s">
+      <c r="F56" s="77" t="s">
         <v>19</v>
       </c>
-      <c r="G56" s="74"/>
-      <c r="H56" s="74"/>
-      <c r="I56" s="74"/>
-      <c r="J56" s="74"/>
-      <c r="K56" s="74"/>
-      <c r="L56" s="74"/>
+      <c r="G56" s="77"/>
+      <c r="H56" s="77"/>
+      <c r="I56" s="77"/>
+      <c r="J56" s="77"/>
+      <c r="K56" s="77"/>
+      <c r="L56" s="77"/>
       <c r="N56" s="16"/>
       <c r="P56" s="21"/>
       <c r="Q56" s="16"/>
@@ -2016,15 +1943,15 @@
       <c r="C57" s="13"/>
       <c r="D57" s="17"/>
       <c r="E57" s="26"/>
-      <c r="F57" s="74" t="s">
+      <c r="F57" s="77" t="s">
         <v>18</v>
       </c>
-      <c r="G57" s="74"/>
-      <c r="H57" s="74"/>
-      <c r="I57" s="74"/>
-      <c r="J57" s="74"/>
-      <c r="K57" s="74"/>
-      <c r="L57" s="74"/>
+      <c r="G57" s="77"/>
+      <c r="H57" s="77"/>
+      <c r="I57" s="77"/>
+      <c r="J57" s="77"/>
+      <c r="K57" s="77"/>
+      <c r="L57" s="77"/>
       <c r="N57" s="16"/>
       <c r="Q57" s="16"/>
       <c r="T57" s="25"/>
@@ -2034,15 +1961,15 @@
       <c r="B58" s="13"/>
       <c r="D58" s="17"/>
       <c r="E58" s="26"/>
-      <c r="F58" s="75" t="s">
+      <c r="F58" s="78" t="s">
         <v>17</v>
       </c>
-      <c r="G58" s="75"/>
-      <c r="H58" s="75"/>
-      <c r="I58" s="75"/>
-      <c r="J58" s="75"/>
-      <c r="K58" s="75"/>
-      <c r="L58" s="75"/>
+      <c r="G58" s="78"/>
+      <c r="H58" s="78"/>
+      <c r="I58" s="78"/>
+      <c r="J58" s="78"/>
+      <c r="K58" s="78"/>
+      <c r="L58" s="78"/>
       <c r="N58" s="16"/>
       <c r="P58" s="21"/>
       <c r="Q58" s="16"/>
@@ -2056,15 +1983,15 @@
       <c r="C59" s="13"/>
       <c r="D59" s="17"/>
       <c r="E59" s="26"/>
-      <c r="F59" s="75" t="s">
+      <c r="F59" s="78" t="s">
         <v>16</v>
       </c>
-      <c r="G59" s="75"/>
-      <c r="H59" s="75"/>
-      <c r="I59" s="75"/>
-      <c r="J59" s="75"/>
-      <c r="K59" s="75"/>
-      <c r="L59" s="75"/>
+      <c r="G59" s="78"/>
+      <c r="H59" s="78"/>
+      <c r="I59" s="78"/>
+      <c r="J59" s="78"/>
+      <c r="K59" s="78"/>
+      <c r="L59" s="78"/>
       <c r="N59" s="16"/>
       <c r="P59"/>
       <c r="Q59" s="16"/>
@@ -2080,15 +2007,15 @@
       <c r="C60" s="13"/>
       <c r="D60" s="17"/>
       <c r="E60" s="26"/>
-      <c r="F60" s="75" t="s">
+      <c r="F60" s="78" t="s">
         <v>14</v>
       </c>
-      <c r="G60" s="75"/>
-      <c r="H60" s="75"/>
-      <c r="I60" s="75"/>
-      <c r="J60" s="75"/>
-      <c r="K60" s="75"/>
-      <c r="L60" s="75"/>
+      <c r="G60" s="78"/>
+      <c r="H60" s="78"/>
+      <c r="I60" s="78"/>
+      <c r="J60" s="78"/>
+      <c r="K60" s="78"/>
+      <c r="L60" s="78"/>
       <c r="N60" s="16"/>
       <c r="P60" s="21"/>
       <c r="Q60" s="16"/>
@@ -2172,11 +2099,11 @@
         <v>10</v>
       </c>
       <c r="G65" s="13"/>
-      <c r="H65" s="70" t="s">
+      <c r="H65" s="74" t="s">
         <v>9</v>
       </c>
-      <c r="I65" s="70"/>
-      <c r="J65" s="70"/>
+      <c r="I65" s="74"/>
+      <c r="J65" s="74"/>
       <c r="N65" s="16"/>
       <c r="P65" s="19"/>
       <c r="Q65" s="16"/>
@@ -2190,11 +2117,11 @@
         <v>8</v>
       </c>
       <c r="G66" s="13"/>
-      <c r="H66" s="70" t="s">
+      <c r="H66" s="74" t="s">
         <v>7</v>
       </c>
-      <c r="I66" s="70"/>
-      <c r="J66" s="70"/>
+      <c r="I66" s="74"/>
+      <c r="J66" s="74"/>
       <c r="N66" s="16"/>
       <c r="P66" s="19"/>
       <c r="Q66" s="18"/>
@@ -2293,19 +2220,19 @@
       <c r="P73" s="6"/>
     </row>
     <row r="74" spans="2:17" ht="19">
-      <c r="B74" s="71" t="s">
+      <c r="B74" s="56" t="s">
         <v>0</v>
       </c>
-      <c r="C74" s="71"/>
-      <c r="D74" s="71"/>
-      <c r="E74" s="71"/>
-      <c r="F74" s="71"/>
-      <c r="G74" s="71"/>
-      <c r="H74" s="71"/>
-      <c r="I74" s="71"/>
-      <c r="J74" s="71"/>
-      <c r="K74" s="71"/>
-      <c r="L74" s="71"/>
+      <c r="C74" s="56"/>
+      <c r="D74" s="56"/>
+      <c r="E74" s="56"/>
+      <c r="F74" s="56"/>
+      <c r="G74" s="56"/>
+      <c r="H74" s="56"/>
+      <c r="I74" s="56"/>
+      <c r="J74" s="56"/>
+      <c r="K74" s="56"/>
+      <c r="L74" s="56"/>
     </row>
     <row r="75" spans="2:17">
       <c r="B75" s="4"/>
@@ -3024,21 +2951,99 @@
     </row>
   </sheetData>
   <mergeCells count="132">
-    <mergeCell ref="J13:L13"/>
-    <mergeCell ref="J14:L14"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="G17:I17"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="H2:L3"/>
-    <mergeCell ref="B5:E12"/>
-    <mergeCell ref="J5:L5"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="J7:L7"/>
-    <mergeCell ref="J8:L8"/>
-    <mergeCell ref="J9:L9"/>
-    <mergeCell ref="J10:L12"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="K17:K18"/>
+    <mergeCell ref="L17:L18"/>
+    <mergeCell ref="E47:E48"/>
+    <mergeCell ref="F47:F48"/>
+    <mergeCell ref="G47:I47"/>
+    <mergeCell ref="J47:J48"/>
+    <mergeCell ref="K47:K48"/>
+    <mergeCell ref="L47:L48"/>
+    <mergeCell ref="G48:I48"/>
+    <mergeCell ref="F45:F46"/>
+    <mergeCell ref="G45:I45"/>
+    <mergeCell ref="J45:J46"/>
+    <mergeCell ref="K45:K46"/>
+    <mergeCell ref="L45:L46"/>
+    <mergeCell ref="G46:I46"/>
+    <mergeCell ref="E45:E46"/>
+    <mergeCell ref="G24:I24"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="J17:J18"/>
+    <mergeCell ref="G18:I18"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="L23:L24"/>
+    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="K25:K26"/>
+    <mergeCell ref="L25:L26"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="K23:K24"/>
+    <mergeCell ref="E43:E44"/>
+    <mergeCell ref="F43:F44"/>
+    <mergeCell ref="G43:I43"/>
+    <mergeCell ref="J43:J44"/>
+    <mergeCell ref="K43:K44"/>
+    <mergeCell ref="G25:I25"/>
+    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="E41:E42"/>
+    <mergeCell ref="G39:I39"/>
+    <mergeCell ref="J39:J40"/>
+    <mergeCell ref="K39:K40"/>
+    <mergeCell ref="L39:L40"/>
+    <mergeCell ref="G40:I40"/>
+    <mergeCell ref="J37:J38"/>
+    <mergeCell ref="K37:K38"/>
+    <mergeCell ref="L37:L38"/>
+    <mergeCell ref="G38:I38"/>
+    <mergeCell ref="E35:E36"/>
+    <mergeCell ref="F35:F36"/>
+    <mergeCell ref="G35:I35"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="H65:J65"/>
+    <mergeCell ref="H66:J66"/>
+    <mergeCell ref="B74:L74"/>
+    <mergeCell ref="E49:E50"/>
+    <mergeCell ref="F49:F50"/>
+    <mergeCell ref="G49:I49"/>
+    <mergeCell ref="G50:I50"/>
+    <mergeCell ref="F56:L56"/>
+    <mergeCell ref="F57:L57"/>
+    <mergeCell ref="F58:L58"/>
+    <mergeCell ref="F59:L59"/>
+    <mergeCell ref="F60:L60"/>
+    <mergeCell ref="L43:L44"/>
+    <mergeCell ref="G44:I44"/>
+    <mergeCell ref="F41:F42"/>
+    <mergeCell ref="G41:I41"/>
+    <mergeCell ref="J41:J42"/>
+    <mergeCell ref="K41:K42"/>
+    <mergeCell ref="L41:L42"/>
+    <mergeCell ref="G42:I42"/>
+    <mergeCell ref="E39:E40"/>
+    <mergeCell ref="F39:F40"/>
+    <mergeCell ref="J35:J36"/>
+    <mergeCell ref="K35:K36"/>
+    <mergeCell ref="L35:L36"/>
+    <mergeCell ref="G36:I36"/>
+    <mergeCell ref="E37:E38"/>
+    <mergeCell ref="F37:F38"/>
+    <mergeCell ref="G37:I37"/>
+    <mergeCell ref="J33:J34"/>
+    <mergeCell ref="K33:K34"/>
+    <mergeCell ref="L33:L34"/>
+    <mergeCell ref="G34:I34"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="G31:I31"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="K31:K32"/>
+    <mergeCell ref="L31:L32"/>
+    <mergeCell ref="G32:I32"/>
+    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="F33:F34"/>
+    <mergeCell ref="G33:I33"/>
     <mergeCell ref="G29:I29"/>
     <mergeCell ref="J29:J30"/>
     <mergeCell ref="K29:K30"/>
@@ -3063,99 +3068,21 @@
     <mergeCell ref="G27:I27"/>
     <mergeCell ref="G28:I28"/>
     <mergeCell ref="E29:E30"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="G31:I31"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="K31:K32"/>
-    <mergeCell ref="L31:L32"/>
-    <mergeCell ref="G32:I32"/>
-    <mergeCell ref="E33:E34"/>
-    <mergeCell ref="F33:F34"/>
-    <mergeCell ref="G33:I33"/>
-    <mergeCell ref="J35:J36"/>
-    <mergeCell ref="K35:K36"/>
-    <mergeCell ref="L35:L36"/>
-    <mergeCell ref="G36:I36"/>
-    <mergeCell ref="E37:E38"/>
-    <mergeCell ref="F37:F38"/>
-    <mergeCell ref="G37:I37"/>
-    <mergeCell ref="J33:J34"/>
-    <mergeCell ref="K33:K34"/>
-    <mergeCell ref="L33:L34"/>
-    <mergeCell ref="G34:I34"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="F21:F22"/>
-    <mergeCell ref="H65:J65"/>
-    <mergeCell ref="H66:J66"/>
-    <mergeCell ref="B74:L74"/>
-    <mergeCell ref="E49:E50"/>
-    <mergeCell ref="F49:F50"/>
-    <mergeCell ref="G49:I49"/>
-    <mergeCell ref="G50:I50"/>
-    <mergeCell ref="F56:L56"/>
-    <mergeCell ref="F57:L57"/>
-    <mergeCell ref="F58:L58"/>
-    <mergeCell ref="F59:L59"/>
-    <mergeCell ref="F60:L60"/>
-    <mergeCell ref="L43:L44"/>
-    <mergeCell ref="G44:I44"/>
-    <mergeCell ref="F41:F42"/>
-    <mergeCell ref="G41:I41"/>
-    <mergeCell ref="J41:J42"/>
-    <mergeCell ref="K41:K42"/>
-    <mergeCell ref="L41:L42"/>
-    <mergeCell ref="G42:I42"/>
-    <mergeCell ref="E39:E40"/>
-    <mergeCell ref="F39:F40"/>
-    <mergeCell ref="K25:K26"/>
-    <mergeCell ref="L25:L26"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="K23:K24"/>
-    <mergeCell ref="E43:E44"/>
-    <mergeCell ref="F43:F44"/>
-    <mergeCell ref="G43:I43"/>
-    <mergeCell ref="J43:J44"/>
-    <mergeCell ref="K43:K44"/>
-    <mergeCell ref="G25:I25"/>
-    <mergeCell ref="G26:I26"/>
-    <mergeCell ref="E41:E42"/>
-    <mergeCell ref="G39:I39"/>
-    <mergeCell ref="J39:J40"/>
-    <mergeCell ref="K39:K40"/>
-    <mergeCell ref="L39:L40"/>
-    <mergeCell ref="G40:I40"/>
-    <mergeCell ref="J37:J38"/>
-    <mergeCell ref="K37:K38"/>
-    <mergeCell ref="L37:L38"/>
-    <mergeCell ref="G38:I38"/>
-    <mergeCell ref="E35:E36"/>
-    <mergeCell ref="F35:F36"/>
-    <mergeCell ref="G35:I35"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="K17:K18"/>
-    <mergeCell ref="L17:L18"/>
-    <mergeCell ref="E47:E48"/>
-    <mergeCell ref="F47:F48"/>
-    <mergeCell ref="G47:I47"/>
-    <mergeCell ref="J47:J48"/>
-    <mergeCell ref="K47:K48"/>
-    <mergeCell ref="L47:L48"/>
-    <mergeCell ref="G48:I48"/>
-    <mergeCell ref="F45:F46"/>
-    <mergeCell ref="G45:I45"/>
-    <mergeCell ref="J45:J46"/>
-    <mergeCell ref="K45:K46"/>
-    <mergeCell ref="L45:L46"/>
-    <mergeCell ref="G46:I46"/>
-    <mergeCell ref="E45:E46"/>
-    <mergeCell ref="G24:I24"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="J17:J18"/>
-    <mergeCell ref="G18:I18"/>
-    <mergeCell ref="J19:J20"/>
-    <mergeCell ref="L23:L24"/>
-    <mergeCell ref="J25:J26"/>
+    <mergeCell ref="J13:L13"/>
+    <mergeCell ref="J14:L14"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="H2:L3"/>
+    <mergeCell ref="B5:E12"/>
+    <mergeCell ref="J5:L5"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="J8:L8"/>
+    <mergeCell ref="J9:L9"/>
+    <mergeCell ref="J10:L12"/>
   </mergeCells>
   <phoneticPr fontId="30" type="noConversion"/>
   <pageMargins left="0.75" right="0" top="0.75" bottom="0.25" header="0.3" footer="0"/>

</xml_diff>

<commit_message>
apply area-based cost only to material-priced quote items
</commit_message>
<xml_diff>
--- a/app/assets/quote_template.xlsx
+++ b/app/assets/quote_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kevinkao/Documents/software building/b2b-quotation-project/b2b-quotation-system-backend/app/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB5E682C-F37F-0D40-87EF-2014CDD72CA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5A04F36-A916-3D49-B61B-8AEC5164650A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="27040" windowHeight="16940" xr2:uid="{3E340372-419D-D74C-8630-F9BDE50D3BA2}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t>Address  臺北市信義區基隆路一段206號18樓   /   Tel  02 7709 7001  /  Cellphone  0988 697 165  /   Tax Number  82817282</t>
   </si>
@@ -156,31 +156,16 @@
     <t>項目名稱</t>
   </si>
   <si>
-    <t>高孟涵 Echo</t>
-  </si>
-  <si>
     <t>聯絡人</t>
   </si>
   <si>
-    <t>0287707072</t>
-  </si>
-  <si>
     <t>聯絡電話</t>
   </si>
   <si>
-    <t>70754038</t>
-  </si>
-  <si>
     <t>統一編號</t>
   </si>
   <si>
-    <t>新加坡商網達先進科技有限公司台灣分公司</t>
-  </si>
-  <si>
     <t>公司名稱</t>
-  </si>
-  <si>
-    <t>2025. 12. 24</t>
   </si>
   <si>
     <t>時間</t>
@@ -593,6 +578,87 @@
     <xf numFmtId="41" fontId="20" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="20" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="20" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="21" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="41" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -608,18 +674,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -631,78 +688,6 @@
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="21" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="180" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="20" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="20" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1205,10 +1190,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:18">
-      <c r="L1" s="60" t="s">
-        <v>42</v>
-      </c>
-      <c r="M1" s="60"/>
+      <c r="L1" s="84" t="s">
+        <v>37</v>
+      </c>
+      <c r="M1" s="84"/>
     </row>
     <row r="2" spans="2:18" ht="21" customHeight="1">
       <c r="B2" s="13"/>
@@ -1217,13 +1202,13 @@
       <c r="E2" s="13"/>
       <c r="F2" s="5"/>
       <c r="G2" s="13"/>
-      <c r="H2" s="61" t="s">
-        <v>41</v>
-      </c>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
-      <c r="K2" s="62"/>
-      <c r="L2" s="62"/>
+      <c r="H2" s="85" t="s">
+        <v>36</v>
+      </c>
+      <c r="I2" s="86"/>
+      <c r="J2" s="86"/>
+      <c r="K2" s="86"/>
+      <c r="L2" s="86"/>
     </row>
     <row r="3" spans="2:18" ht="21" customHeight="1">
       <c r="B3" s="13"/>
@@ -1232,11 +1217,11 @@
       <c r="E3" s="13"/>
       <c r="F3" s="5"/>
       <c r="G3" s="13"/>
-      <c r="H3" s="62"/>
-      <c r="I3" s="62"/>
-      <c r="J3" s="62"/>
-      <c r="K3" s="62"/>
-      <c r="L3" s="62"/>
+      <c r="H3" s="86"/>
+      <c r="I3" s="86"/>
+      <c r="J3" s="86"/>
+      <c r="K3" s="86"/>
+      <c r="L3" s="86"/>
     </row>
     <row r="4" spans="2:18" ht="34" customHeight="1">
       <c r="B4" s="13"/>
@@ -1250,133 +1235,123 @@
       <c r="J4" s="5"/>
     </row>
     <row r="5" spans="2:18" ht="21">
-      <c r="B5" s="56"/>
-      <c r="C5" s="56"/>
-      <c r="D5" s="56"/>
-      <c r="E5" s="56"/>
+      <c r="B5" s="70"/>
+      <c r="C5" s="70"/>
+      <c r="D5" s="70"/>
+      <c r="E5" s="70"/>
       <c r="F5" s="5"/>
       <c r="I5" s="48" t="s">
-        <v>40</v>
-      </c>
-      <c r="J5" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="K5" s="53"/>
-      <c r="L5" s="53"/>
+        <v>35</v>
+      </c>
+      <c r="J5" s="80"/>
+      <c r="K5" s="80"/>
+      <c r="L5" s="80"/>
     </row>
     <row r="6" spans="2:18" ht="26" customHeight="1">
-      <c r="B6" s="56"/>
-      <c r="C6" s="56"/>
-      <c r="D6" s="56"/>
-      <c r="E6" s="56"/>
+      <c r="B6" s="70"/>
+      <c r="C6" s="70"/>
+      <c r="D6" s="70"/>
+      <c r="E6" s="70"/>
       <c r="F6" s="5"/>
       <c r="I6" s="48" t="s">
-        <v>38</v>
-      </c>
-      <c r="J6" s="53" t="s">
-        <v>37</v>
-      </c>
-      <c r="K6" s="53"/>
-      <c r="L6" s="53"/>
+        <v>34</v>
+      </c>
+      <c r="J6" s="80"/>
+      <c r="K6" s="80"/>
+      <c r="L6" s="80"/>
     </row>
     <row r="7" spans="2:18" ht="26" customHeight="1">
-      <c r="B7" s="56"/>
-      <c r="C7" s="56"/>
-      <c r="D7" s="56"/>
-      <c r="E7" s="56"/>
+      <c r="B7" s="70"/>
+      <c r="C7" s="70"/>
+      <c r="D7" s="70"/>
+      <c r="E7" s="70"/>
       <c r="F7" s="5"/>
       <c r="I7" s="48" t="s">
-        <v>36</v>
-      </c>
-      <c r="J7" s="53" t="s">
-        <v>35</v>
-      </c>
-      <c r="K7" s="53"/>
-      <c r="L7" s="53"/>
+        <v>33</v>
+      </c>
+      <c r="J7" s="80"/>
+      <c r="K7" s="80"/>
+      <c r="L7" s="80"/>
     </row>
     <row r="8" spans="2:18" ht="26" customHeight="1">
-      <c r="B8" s="56"/>
-      <c r="C8" s="56"/>
-      <c r="D8" s="56"/>
-      <c r="E8" s="56"/>
+      <c r="B8" s="70"/>
+      <c r="C8" s="70"/>
+      <c r="D8" s="70"/>
+      <c r="E8" s="70"/>
       <c r="F8" s="5"/>
       <c r="H8" s="8"/>
       <c r="I8" s="48" t="s">
-        <v>34</v>
-      </c>
-      <c r="J8" s="53" t="s">
-        <v>33</v>
-      </c>
-      <c r="K8" s="53"/>
-      <c r="L8" s="53"/>
+        <v>32</v>
+      </c>
+      <c r="J8" s="80"/>
+      <c r="K8" s="80"/>
+      <c r="L8" s="80"/>
     </row>
     <row r="9" spans="2:18" ht="21">
-      <c r="B9" s="56"/>
-      <c r="C9" s="56"/>
-      <c r="D9" s="56"/>
-      <c r="E9" s="56"/>
+      <c r="B9" s="70"/>
+      <c r="C9" s="70"/>
+      <c r="D9" s="70"/>
+      <c r="E9" s="70"/>
       <c r="F9" s="5"/>
       <c r="I9" s="48" t="s">
-        <v>32</v>
-      </c>
-      <c r="J9" s="53" t="s">
         <v>31</v>
       </c>
-      <c r="K9" s="53"/>
-      <c r="L9" s="53"/>
+      <c r="J9" s="80"/>
+      <c r="K9" s="80"/>
+      <c r="L9" s="80"/>
     </row>
     <row r="10" spans="2:18" ht="28" customHeight="1">
-      <c r="B10" s="56"/>
-      <c r="C10" s="56"/>
-      <c r="D10" s="56"/>
-      <c r="E10" s="56"/>
+      <c r="B10" s="70"/>
+      <c r="C10" s="70"/>
+      <c r="D10" s="70"/>
+      <c r="E10" s="70"/>
       <c r="F10" s="5"/>
       <c r="I10" s="48" t="s">
         <v>30</v>
       </c>
-      <c r="J10" s="63"/>
-      <c r="K10" s="63"/>
-      <c r="L10" s="63"/>
+      <c r="J10" s="87"/>
+      <c r="K10" s="87"/>
+      <c r="L10" s="87"/>
     </row>
     <row r="11" spans="2:18" ht="21" customHeight="1">
-      <c r="B11" s="56"/>
-      <c r="C11" s="56"/>
-      <c r="D11" s="56"/>
-      <c r="E11" s="56"/>
+      <c r="B11" s="70"/>
+      <c r="C11" s="70"/>
+      <c r="D11" s="70"/>
+      <c r="E11" s="70"/>
       <c r="F11" s="5"/>
       <c r="G11" s="13"/>
       <c r="H11" s="8"/>
       <c r="I11" s="13"/>
-      <c r="J11" s="63"/>
-      <c r="K11" s="63"/>
-      <c r="L11" s="63"/>
+      <c r="J11" s="87"/>
+      <c r="K11" s="87"/>
+      <c r="L11" s="87"/>
     </row>
     <row r="12" spans="2:18" ht="21" customHeight="1">
-      <c r="B12" s="56"/>
-      <c r="C12" s="56"/>
-      <c r="D12" s="56"/>
-      <c r="E12" s="56"/>
-      <c r="J12" s="63"/>
-      <c r="K12" s="63"/>
-      <c r="L12" s="63"/>
+      <c r="B12" s="70"/>
+      <c r="C12" s="70"/>
+      <c r="D12" s="70"/>
+      <c r="E12" s="70"/>
+      <c r="J12" s="87"/>
+      <c r="K12" s="87"/>
+      <c r="L12" s="87"/>
     </row>
     <row r="13" spans="2:18" ht="21">
       <c r="B13" s="13"/>
       <c r="C13" s="13"/>
       <c r="D13" s="13"/>
       <c r="I13" s="48"/>
-      <c r="J13" s="51"/>
-      <c r="K13" s="52"/>
-      <c r="L13" s="52"/>
+      <c r="J13" s="78"/>
+      <c r="K13" s="79"/>
+      <c r="L13" s="79"/>
     </row>
     <row r="14" spans="2:18" ht="21" customHeight="1">
       <c r="B14" s="13"/>
       <c r="C14" s="13"/>
       <c r="D14" s="13"/>
       <c r="I14" s="48"/>
-      <c r="J14" s="53"/>
-      <c r="K14" s="53"/>
-      <c r="L14" s="53"/>
+      <c r="J14" s="80"/>
+      <c r="K14" s="80"/>
+      <c r="L14" s="80"/>
     </row>
     <row r="15" spans="2:18" ht="21" customHeight="1">
       <c r="B15" s="13"/>
@@ -1397,11 +1372,11 @@
       <c r="F16" s="45" t="s">
         <v>28</v>
       </c>
-      <c r="G16" s="54" t="s">
+      <c r="G16" s="81" t="s">
         <v>27</v>
       </c>
-      <c r="H16" s="54"/>
-      <c r="I16" s="54"/>
+      <c r="H16" s="81"/>
+      <c r="I16" s="81"/>
       <c r="J16" s="45" t="s">
         <v>26</v>
       </c>
@@ -1419,16 +1394,16 @@
       <c r="B17" s="13"/>
       <c r="C17" s="13"/>
       <c r="D17" s="13"/>
-      <c r="E17" s="55">
+      <c r="E17" s="82">
         <v>1</v>
       </c>
-      <c r="F17" s="57"/>
-      <c r="G17" s="59"/>
-      <c r="H17" s="59"/>
-      <c r="I17" s="59"/>
-      <c r="J17" s="87"/>
-      <c r="K17" s="85"/>
-      <c r="L17" s="85">
+      <c r="F17" s="83"/>
+      <c r="G17" s="67"/>
+      <c r="H17" s="67"/>
+      <c r="I17" s="67"/>
+      <c r="J17" s="64"/>
+      <c r="K17" s="53"/>
+      <c r="L17" s="53">
         <f>J17*K17</f>
         <v>0</v>
       </c>
@@ -1438,28 +1413,28 @@
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
-      <c r="E18" s="56"/>
-      <c r="F18" s="58"/>
-      <c r="G18" s="68"/>
-      <c r="H18" s="68"/>
-      <c r="I18" s="68"/>
-      <c r="J18" s="65"/>
-      <c r="K18" s="86"/>
-      <c r="L18" s="86"/>
+      <c r="E18" s="70"/>
+      <c r="F18" s="52"/>
+      <c r="G18" s="61"/>
+      <c r="H18" s="61"/>
+      <c r="I18" s="61"/>
+      <c r="J18" s="63"/>
+      <c r="K18" s="54"/>
+      <c r="L18" s="54"/>
       <c r="O18" s="43"/>
     </row>
     <row r="19" spans="2:19" ht="21" customHeight="1">
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
       <c r="D19" s="13"/>
-      <c r="E19" s="69">
+      <c r="E19" s="71">
         <v>2</v>
       </c>
-      <c r="F19" s="71"/>
-      <c r="G19" s="59"/>
-      <c r="H19" s="59"/>
-      <c r="I19" s="59"/>
-      <c r="J19" s="64"/>
+      <c r="F19" s="51"/>
+      <c r="G19" s="67"/>
+      <c r="H19" s="67"/>
+      <c r="I19" s="67"/>
+      <c r="J19" s="62"/>
       <c r="K19" s="49"/>
       <c r="L19" s="49"/>
       <c r="Q19" s="42"/>
@@ -1468,12 +1443,12 @@
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
-      <c r="E20" s="70"/>
-      <c r="F20" s="58"/>
-      <c r="G20" s="68"/>
-      <c r="H20" s="68"/>
-      <c r="I20" s="68"/>
-      <c r="J20" s="65"/>
+      <c r="E20" s="72"/>
+      <c r="F20" s="52"/>
+      <c r="G20" s="61"/>
+      <c r="H20" s="61"/>
+      <c r="I20" s="61"/>
+      <c r="J20" s="63"/>
       <c r="K20" s="49"/>
       <c r="L20" s="49"/>
     </row>
@@ -1481,14 +1456,14 @@
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
-      <c r="E21" s="69">
+      <c r="E21" s="71">
         <v>2</v>
       </c>
-      <c r="F21" s="71"/>
-      <c r="G21" s="59"/>
-      <c r="H21" s="59"/>
-      <c r="I21" s="59"/>
-      <c r="J21" s="64"/>
+      <c r="F21" s="51"/>
+      <c r="G21" s="67"/>
+      <c r="H21" s="67"/>
+      <c r="I21" s="67"/>
+      <c r="J21" s="62"/>
       <c r="K21" s="49"/>
       <c r="L21" s="49"/>
       <c r="Q21" s="42"/>
@@ -1497,333 +1472,333 @@
       <c r="B22" s="13"/>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
-      <c r="E22" s="70"/>
-      <c r="F22" s="58"/>
-      <c r="G22" s="68"/>
-      <c r="H22" s="68"/>
-      <c r="I22" s="68"/>
-      <c r="J22" s="65"/>
+      <c r="E22" s="72"/>
+      <c r="F22" s="52"/>
+      <c r="G22" s="61"/>
+      <c r="H22" s="61"/>
+      <c r="I22" s="61"/>
+      <c r="J22" s="63"/>
       <c r="K22" s="50"/>
       <c r="L22" s="50"/>
       <c r="P22"/>
     </row>
     <row r="23" spans="2:19" ht="21" customHeight="1">
-      <c r="E23" s="56"/>
-      <c r="F23" s="71"/>
-      <c r="G23" s="59"/>
-      <c r="H23" s="59"/>
-      <c r="I23" s="59"/>
-      <c r="J23" s="64"/>
-      <c r="K23" s="66"/>
-      <c r="L23" s="66"/>
+      <c r="E23" s="70"/>
+      <c r="F23" s="51"/>
+      <c r="G23" s="67"/>
+      <c r="H23" s="67"/>
+      <c r="I23" s="67"/>
+      <c r="J23" s="62"/>
+      <c r="K23" s="65"/>
+      <c r="L23" s="65"/>
       <c r="Q23" s="18"/>
       <c r="S23" s="8"/>
     </row>
     <row r="24" spans="2:19" ht="21" customHeight="1">
-      <c r="E24" s="70"/>
-      <c r="F24" s="58"/>
-      <c r="G24" s="68"/>
-      <c r="H24" s="68"/>
-      <c r="I24" s="68"/>
-      <c r="J24" s="65"/>
-      <c r="K24" s="67"/>
-      <c r="L24" s="67"/>
+      <c r="E24" s="72"/>
+      <c r="F24" s="52"/>
+      <c r="G24" s="61"/>
+      <c r="H24" s="61"/>
+      <c r="I24" s="61"/>
+      <c r="J24" s="63"/>
+      <c r="K24" s="66"/>
+      <c r="L24" s="66"/>
       <c r="S24" s="8"/>
     </row>
     <row r="25" spans="2:19" ht="21" customHeight="1">
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
       <c r="D25" s="13"/>
-      <c r="E25" s="56"/>
-      <c r="F25" s="71"/>
-      <c r="G25" s="59"/>
-      <c r="H25" s="59"/>
-      <c r="I25" s="59"/>
-      <c r="J25" s="64"/>
-      <c r="K25" s="66"/>
-      <c r="L25" s="66"/>
+      <c r="E25" s="70"/>
+      <c r="F25" s="51"/>
+      <c r="G25" s="67"/>
+      <c r="H25" s="67"/>
+      <c r="I25" s="67"/>
+      <c r="J25" s="62"/>
+      <c r="K25" s="65"/>
+      <c r="L25" s="65"/>
       <c r="Q25" s="42"/>
     </row>
     <row r="26" spans="2:19" ht="21" customHeight="1">
       <c r="B26" s="13"/>
       <c r="C26" s="13"/>
       <c r="D26" s="13"/>
-      <c r="E26" s="70"/>
-      <c r="F26" s="58"/>
-      <c r="G26" s="68"/>
-      <c r="H26" s="68"/>
-      <c r="I26" s="68"/>
-      <c r="J26" s="65"/>
-      <c r="K26" s="67"/>
-      <c r="L26" s="67"/>
+      <c r="E26" s="72"/>
+      <c r="F26" s="52"/>
+      <c r="G26" s="61"/>
+      <c r="H26" s="61"/>
+      <c r="I26" s="61"/>
+      <c r="J26" s="63"/>
+      <c r="K26" s="66"/>
+      <c r="L26" s="66"/>
     </row>
     <row r="27" spans="2:19" ht="21" customHeight="1">
       <c r="B27" s="13"/>
       <c r="C27" s="13"/>
       <c r="D27" s="13"/>
-      <c r="E27" s="56"/>
-      <c r="F27" s="71"/>
-      <c r="G27" s="59"/>
-      <c r="H27" s="59"/>
-      <c r="I27" s="59"/>
-      <c r="J27" s="64"/>
-      <c r="K27" s="66"/>
-      <c r="L27" s="66"/>
+      <c r="E27" s="70"/>
+      <c r="F27" s="51"/>
+      <c r="G27" s="67"/>
+      <c r="H27" s="67"/>
+      <c r="I27" s="67"/>
+      <c r="J27" s="62"/>
+      <c r="K27" s="65"/>
+      <c r="L27" s="65"/>
       <c r="Q27" s="42"/>
     </row>
     <row r="28" spans="2:19" ht="21" customHeight="1">
       <c r="B28" s="13"/>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
-      <c r="E28" s="70"/>
-      <c r="F28" s="58"/>
-      <c r="G28" s="68"/>
-      <c r="H28" s="68"/>
-      <c r="I28" s="68"/>
-      <c r="J28" s="65"/>
-      <c r="K28" s="67"/>
-      <c r="L28" s="67"/>
+      <c r="E28" s="72"/>
+      <c r="F28" s="52"/>
+      <c r="G28" s="61"/>
+      <c r="H28" s="61"/>
+      <c r="I28" s="61"/>
+      <c r="J28" s="63"/>
+      <c r="K28" s="66"/>
+      <c r="L28" s="66"/>
     </row>
     <row r="29" spans="2:19" ht="21" customHeight="1">
-      <c r="E29" s="56"/>
-      <c r="F29" s="71"/>
-      <c r="G29" s="59"/>
-      <c r="H29" s="59"/>
-      <c r="I29" s="59"/>
-      <c r="J29" s="64"/>
-      <c r="K29" s="66"/>
-      <c r="L29" s="66"/>
+      <c r="E29" s="70"/>
+      <c r="F29" s="51"/>
+      <c r="G29" s="67"/>
+      <c r="H29" s="67"/>
+      <c r="I29" s="67"/>
+      <c r="J29" s="62"/>
+      <c r="K29" s="65"/>
+      <c r="L29" s="65"/>
       <c r="Q29" s="18"/>
       <c r="S29" s="8"/>
     </row>
     <row r="30" spans="2:19" ht="21" customHeight="1">
-      <c r="E30" s="70"/>
-      <c r="F30" s="58"/>
-      <c r="G30" s="68"/>
-      <c r="H30" s="68"/>
-      <c r="I30" s="68"/>
-      <c r="J30" s="65"/>
-      <c r="K30" s="67"/>
-      <c r="L30" s="67"/>
+      <c r="E30" s="72"/>
+      <c r="F30" s="52"/>
+      <c r="G30" s="61"/>
+      <c r="H30" s="61"/>
+      <c r="I30" s="61"/>
+      <c r="J30" s="63"/>
+      <c r="K30" s="66"/>
+      <c r="L30" s="66"/>
       <c r="S30" s="8"/>
     </row>
     <row r="31" spans="2:19" ht="21" customHeight="1">
-      <c r="E31" s="56"/>
-      <c r="F31" s="71"/>
-      <c r="G31" s="59"/>
-      <c r="H31" s="59"/>
-      <c r="I31" s="59"/>
-      <c r="J31" s="64"/>
-      <c r="K31" s="66"/>
-      <c r="L31" s="66"/>
+      <c r="E31" s="70"/>
+      <c r="F31" s="51"/>
+      <c r="G31" s="67"/>
+      <c r="H31" s="67"/>
+      <c r="I31" s="67"/>
+      <c r="J31" s="62"/>
+      <c r="K31" s="65"/>
+      <c r="L31" s="65"/>
       <c r="Q31" s="18"/>
       <c r="S31" s="8"/>
     </row>
     <row r="32" spans="2:19" ht="21" customHeight="1">
-      <c r="E32" s="70"/>
-      <c r="F32" s="58"/>
-      <c r="G32" s="68"/>
-      <c r="H32" s="68"/>
-      <c r="I32" s="68"/>
-      <c r="J32" s="65"/>
-      <c r="K32" s="67"/>
-      <c r="L32" s="67"/>
+      <c r="E32" s="72"/>
+      <c r="F32" s="52"/>
+      <c r="G32" s="61"/>
+      <c r="H32" s="61"/>
+      <c r="I32" s="61"/>
+      <c r="J32" s="63"/>
+      <c r="K32" s="66"/>
+      <c r="L32" s="66"/>
       <c r="S32" s="8"/>
     </row>
     <row r="33" spans="2:19" ht="21" customHeight="1">
-      <c r="E33" s="56"/>
-      <c r="F33" s="71"/>
-      <c r="G33" s="59"/>
-      <c r="H33" s="59"/>
-      <c r="I33" s="59"/>
-      <c r="J33" s="64"/>
-      <c r="K33" s="72"/>
-      <c r="L33" s="72"/>
+      <c r="E33" s="70"/>
+      <c r="F33" s="51"/>
+      <c r="G33" s="67"/>
+      <c r="H33" s="67"/>
+      <c r="I33" s="67"/>
+      <c r="J33" s="62"/>
+      <c r="K33" s="68"/>
+      <c r="L33" s="68"/>
       <c r="Q33" s="18"/>
       <c r="S33" s="8"/>
     </row>
     <row r="34" spans="2:19" ht="21" customHeight="1">
-      <c r="E34" s="56"/>
-      <c r="F34" s="71"/>
-      <c r="G34" s="73"/>
-      <c r="H34" s="73"/>
-      <c r="I34" s="73"/>
-      <c r="J34" s="64"/>
-      <c r="K34" s="72"/>
-      <c r="L34" s="72"/>
+      <c r="E34" s="70"/>
+      <c r="F34" s="51"/>
+      <c r="G34" s="69"/>
+      <c r="H34" s="69"/>
+      <c r="I34" s="69"/>
+      <c r="J34" s="62"/>
+      <c r="K34" s="68"/>
+      <c r="L34" s="68"/>
       <c r="S34" s="8"/>
     </row>
     <row r="35" spans="2:19" ht="21" customHeight="1">
       <c r="B35" s="13"/>
       <c r="C35" s="13"/>
       <c r="D35" s="13"/>
-      <c r="E35" s="56"/>
-      <c r="F35" s="71"/>
-      <c r="G35" s="59"/>
-      <c r="H35" s="59"/>
-      <c r="I35" s="59"/>
-      <c r="J35" s="64"/>
-      <c r="K35" s="72"/>
-      <c r="L35" s="72"/>
+      <c r="E35" s="70"/>
+      <c r="F35" s="51"/>
+      <c r="G35" s="67"/>
+      <c r="H35" s="67"/>
+      <c r="I35" s="67"/>
+      <c r="J35" s="62"/>
+      <c r="K35" s="68"/>
+      <c r="L35" s="68"/>
       <c r="Q35" s="42"/>
     </row>
     <row r="36" spans="2:19" ht="23" customHeight="1">
       <c r="B36" s="13"/>
       <c r="C36" s="13"/>
       <c r="D36" s="13"/>
-      <c r="E36" s="56"/>
-      <c r="F36" s="71"/>
-      <c r="G36" s="73"/>
-      <c r="H36" s="73"/>
-      <c r="I36" s="73"/>
-      <c r="J36" s="64"/>
-      <c r="K36" s="72"/>
-      <c r="L36" s="72"/>
+      <c r="E36" s="70"/>
+      <c r="F36" s="51"/>
+      <c r="G36" s="69"/>
+      <c r="H36" s="69"/>
+      <c r="I36" s="69"/>
+      <c r="J36" s="62"/>
+      <c r="K36" s="68"/>
+      <c r="L36" s="68"/>
     </row>
     <row r="37" spans="2:19" ht="21" customHeight="1">
-      <c r="E37" s="56"/>
-      <c r="F37" s="71"/>
-      <c r="G37" s="59"/>
-      <c r="H37" s="59"/>
-      <c r="I37" s="59"/>
-      <c r="J37" s="64"/>
-      <c r="K37" s="72"/>
-      <c r="L37" s="72"/>
+      <c r="E37" s="70"/>
+      <c r="F37" s="51"/>
+      <c r="G37" s="67"/>
+      <c r="H37" s="67"/>
+      <c r="I37" s="67"/>
+      <c r="J37" s="62"/>
+      <c r="K37" s="68"/>
+      <c r="L37" s="68"/>
       <c r="Q37" s="18"/>
       <c r="S37" s="8"/>
     </row>
     <row r="38" spans="2:19" ht="21" customHeight="1">
-      <c r="E38" s="56"/>
-      <c r="F38" s="71"/>
-      <c r="G38" s="73"/>
-      <c r="H38" s="73"/>
-      <c r="I38" s="73"/>
-      <c r="J38" s="64"/>
-      <c r="K38" s="72"/>
-      <c r="L38" s="72"/>
+      <c r="E38" s="70"/>
+      <c r="F38" s="51"/>
+      <c r="G38" s="69"/>
+      <c r="H38" s="69"/>
+      <c r="I38" s="69"/>
+      <c r="J38" s="62"/>
+      <c r="K38" s="68"/>
+      <c r="L38" s="68"/>
       <c r="S38" s="8"/>
     </row>
     <row r="39" spans="2:19" ht="21" customHeight="1">
-      <c r="E39" s="84"/>
-      <c r="F39" s="81"/>
-      <c r="G39" s="82"/>
-      <c r="H39" s="82"/>
-      <c r="I39" s="82"/>
-      <c r="J39" s="83"/>
-      <c r="K39" s="79"/>
-      <c r="L39" s="79"/>
+      <c r="E39" s="55"/>
+      <c r="F39" s="56"/>
+      <c r="G39" s="57"/>
+      <c r="H39" s="57"/>
+      <c r="I39" s="57"/>
+      <c r="J39" s="58"/>
+      <c r="K39" s="59"/>
+      <c r="L39" s="59"/>
       <c r="Q39" s="18"/>
       <c r="S39" s="8"/>
     </row>
     <row r="40" spans="2:19" ht="21" customHeight="1">
-      <c r="E40" s="84"/>
-      <c r="F40" s="81"/>
-      <c r="G40" s="80"/>
-      <c r="H40" s="80"/>
-      <c r="I40" s="80"/>
-      <c r="J40" s="83"/>
-      <c r="K40" s="79"/>
-      <c r="L40" s="79"/>
+      <c r="E40" s="55"/>
+      <c r="F40" s="56"/>
+      <c r="G40" s="60"/>
+      <c r="H40" s="60"/>
+      <c r="I40" s="60"/>
+      <c r="J40" s="58"/>
+      <c r="K40" s="59"/>
+      <c r="L40" s="59"/>
       <c r="S40" s="8"/>
     </row>
     <row r="41" spans="2:19" ht="21" customHeight="1">
-      <c r="E41" s="84"/>
-      <c r="F41" s="81"/>
-      <c r="G41" s="82"/>
-      <c r="H41" s="82"/>
-      <c r="I41" s="82"/>
-      <c r="J41" s="83"/>
-      <c r="K41" s="79"/>
-      <c r="L41" s="79"/>
+      <c r="E41" s="55"/>
+      <c r="F41" s="56"/>
+      <c r="G41" s="57"/>
+      <c r="H41" s="57"/>
+      <c r="I41" s="57"/>
+      <c r="J41" s="58"/>
+      <c r="K41" s="59"/>
+      <c r="L41" s="59"/>
       <c r="Q41" s="18"/>
       <c r="S41" s="8"/>
     </row>
     <row r="42" spans="2:19" ht="21" customHeight="1">
-      <c r="E42" s="84"/>
-      <c r="F42" s="81"/>
-      <c r="G42" s="80"/>
-      <c r="H42" s="80"/>
-      <c r="I42" s="80"/>
-      <c r="J42" s="83"/>
-      <c r="K42" s="79"/>
-      <c r="L42" s="79"/>
+      <c r="E42" s="55"/>
+      <c r="F42" s="56"/>
+      <c r="G42" s="60"/>
+      <c r="H42" s="60"/>
+      <c r="I42" s="60"/>
+      <c r="J42" s="58"/>
+      <c r="K42" s="59"/>
+      <c r="L42" s="59"/>
       <c r="S42" s="8"/>
     </row>
     <row r="43" spans="2:19" ht="21" customHeight="1">
-      <c r="E43" s="84"/>
-      <c r="F43" s="81"/>
-      <c r="G43" s="82"/>
-      <c r="H43" s="82"/>
-      <c r="I43" s="82"/>
-      <c r="J43" s="83"/>
-      <c r="K43" s="79"/>
-      <c r="L43" s="79"/>
+      <c r="E43" s="55"/>
+      <c r="F43" s="56"/>
+      <c r="G43" s="57"/>
+      <c r="H43" s="57"/>
+      <c r="I43" s="57"/>
+      <c r="J43" s="58"/>
+      <c r="K43" s="59"/>
+      <c r="L43" s="59"/>
       <c r="Q43" s="18"/>
       <c r="S43" s="8"/>
     </row>
     <row r="44" spans="2:19" ht="21" customHeight="1">
-      <c r="E44" s="84"/>
-      <c r="F44" s="81"/>
-      <c r="G44" s="80"/>
-      <c r="H44" s="80"/>
-      <c r="I44" s="80"/>
-      <c r="J44" s="83"/>
-      <c r="K44" s="79"/>
-      <c r="L44" s="79"/>
+      <c r="E44" s="55"/>
+      <c r="F44" s="56"/>
+      <c r="G44" s="60"/>
+      <c r="H44" s="60"/>
+      <c r="I44" s="60"/>
+      <c r="J44" s="58"/>
+      <c r="K44" s="59"/>
+      <c r="L44" s="59"/>
       <c r="S44" s="8"/>
     </row>
     <row r="45" spans="2:19" ht="21" customHeight="1">
-      <c r="E45" s="84"/>
-      <c r="F45" s="81"/>
-      <c r="G45" s="82"/>
-      <c r="H45" s="82"/>
-      <c r="I45" s="82"/>
-      <c r="J45" s="83"/>
-      <c r="K45" s="79"/>
-      <c r="L45" s="79"/>
+      <c r="E45" s="55"/>
+      <c r="F45" s="56"/>
+      <c r="G45" s="57"/>
+      <c r="H45" s="57"/>
+      <c r="I45" s="57"/>
+      <c r="J45" s="58"/>
+      <c r="K45" s="59"/>
+      <c r="L45" s="59"/>
       <c r="Q45" s="18"/>
       <c r="S45" s="8"/>
     </row>
     <row r="46" spans="2:19" ht="21" customHeight="1">
-      <c r="E46" s="84"/>
-      <c r="F46" s="81"/>
-      <c r="G46" s="80"/>
-      <c r="H46" s="80"/>
-      <c r="I46" s="80"/>
-      <c r="J46" s="83"/>
-      <c r="K46" s="79"/>
-      <c r="L46" s="79"/>
+      <c r="E46" s="55"/>
+      <c r="F46" s="56"/>
+      <c r="G46" s="60"/>
+      <c r="H46" s="60"/>
+      <c r="I46" s="60"/>
+      <c r="J46" s="58"/>
+      <c r="K46" s="59"/>
+      <c r="L46" s="59"/>
       <c r="S46" s="8"/>
     </row>
     <row r="47" spans="2:19" ht="21" customHeight="1">
-      <c r="E47" s="84"/>
-      <c r="F47" s="81"/>
-      <c r="G47" s="82"/>
-      <c r="H47" s="82"/>
-      <c r="I47" s="82"/>
-      <c r="J47" s="83"/>
-      <c r="K47" s="79"/>
-      <c r="L47" s="79"/>
+      <c r="E47" s="55"/>
+      <c r="F47" s="56"/>
+      <c r="G47" s="57"/>
+      <c r="H47" s="57"/>
+      <c r="I47" s="57"/>
+      <c r="J47" s="58"/>
+      <c r="K47" s="59"/>
+      <c r="L47" s="59"/>
       <c r="Q47" s="18"/>
       <c r="S47" s="8"/>
     </row>
     <row r="48" spans="2:19" ht="21" customHeight="1">
-      <c r="E48" s="84"/>
-      <c r="F48" s="81"/>
-      <c r="G48" s="80"/>
-      <c r="H48" s="80"/>
-      <c r="I48" s="80"/>
-      <c r="J48" s="83"/>
-      <c r="K48" s="79"/>
-      <c r="L48" s="79"/>
+      <c r="E48" s="55"/>
+      <c r="F48" s="56"/>
+      <c r="G48" s="60"/>
+      <c r="H48" s="60"/>
+      <c r="I48" s="60"/>
+      <c r="J48" s="58"/>
+      <c r="K48" s="59"/>
+      <c r="L48" s="59"/>
       <c r="S48" s="8"/>
     </row>
     <row r="49" spans="2:21" ht="21" customHeight="1">
-      <c r="E49" s="56"/>
-      <c r="F49" s="71"/>
-      <c r="G49" s="75"/>
-      <c r="H49" s="75"/>
-      <c r="I49" s="75"/>
+      <c r="E49" s="70"/>
+      <c r="F49" s="51"/>
+      <c r="G49" s="74"/>
+      <c r="H49" s="74"/>
+      <c r="I49" s="74"/>
       <c r="J49" s="41"/>
       <c r="K49" s="40" t="s">
         <v>23</v>
@@ -1838,11 +1813,11 @@
       <c r="S49" s="8"/>
     </row>
     <row r="50" spans="2:21" ht="21" customHeight="1">
-      <c r="E50" s="56"/>
-      <c r="F50" s="71"/>
-      <c r="G50" s="76"/>
-      <c r="H50" s="76"/>
-      <c r="I50" s="76"/>
+      <c r="E50" s="70"/>
+      <c r="F50" s="51"/>
+      <c r="G50" s="75"/>
+      <c r="H50" s="75"/>
+      <c r="I50" s="75"/>
       <c r="J50" s="38"/>
       <c r="K50" s="37" t="s">
         <v>22</v>
@@ -1921,15 +1896,15 @@
         <v>20</v>
       </c>
       <c r="E56" s="28"/>
-      <c r="F56" s="77" t="s">
+      <c r="F56" s="76" t="s">
         <v>19</v>
       </c>
-      <c r="G56" s="77"/>
-      <c r="H56" s="77"/>
-      <c r="I56" s="77"/>
-      <c r="J56" s="77"/>
-      <c r="K56" s="77"/>
-      <c r="L56" s="77"/>
+      <c r="G56" s="76"/>
+      <c r="H56" s="76"/>
+      <c r="I56" s="76"/>
+      <c r="J56" s="76"/>
+      <c r="K56" s="76"/>
+      <c r="L56" s="76"/>
       <c r="N56" s="16"/>
       <c r="P56" s="21"/>
       <c r="Q56" s="16"/>
@@ -1943,15 +1918,15 @@
       <c r="C57" s="13"/>
       <c r="D57" s="17"/>
       <c r="E57" s="26"/>
-      <c r="F57" s="77" t="s">
+      <c r="F57" s="76" t="s">
         <v>18</v>
       </c>
-      <c r="G57" s="77"/>
-      <c r="H57" s="77"/>
-      <c r="I57" s="77"/>
-      <c r="J57" s="77"/>
-      <c r="K57" s="77"/>
-      <c r="L57" s="77"/>
+      <c r="G57" s="76"/>
+      <c r="H57" s="76"/>
+      <c r="I57" s="76"/>
+      <c r="J57" s="76"/>
+      <c r="K57" s="76"/>
+      <c r="L57" s="76"/>
       <c r="N57" s="16"/>
       <c r="Q57" s="16"/>
       <c r="T57" s="25"/>
@@ -1961,15 +1936,15 @@
       <c r="B58" s="13"/>
       <c r="D58" s="17"/>
       <c r="E58" s="26"/>
-      <c r="F58" s="78" t="s">
+      <c r="F58" s="77" t="s">
         <v>17</v>
       </c>
-      <c r="G58" s="78"/>
-      <c r="H58" s="78"/>
-      <c r="I58" s="78"/>
-      <c r="J58" s="78"/>
-      <c r="K58" s="78"/>
-      <c r="L58" s="78"/>
+      <c r="G58" s="77"/>
+      <c r="H58" s="77"/>
+      <c r="I58" s="77"/>
+      <c r="J58" s="77"/>
+      <c r="K58" s="77"/>
+      <c r="L58" s="77"/>
       <c r="N58" s="16"/>
       <c r="P58" s="21"/>
       <c r="Q58" s="16"/>
@@ -1983,15 +1958,15 @@
       <c r="C59" s="13"/>
       <c r="D59" s="17"/>
       <c r="E59" s="26"/>
-      <c r="F59" s="78" t="s">
+      <c r="F59" s="77" t="s">
         <v>16</v>
       </c>
-      <c r="G59" s="78"/>
-      <c r="H59" s="78"/>
-      <c r="I59" s="78"/>
-      <c r="J59" s="78"/>
-      <c r="K59" s="78"/>
-      <c r="L59" s="78"/>
+      <c r="G59" s="77"/>
+      <c r="H59" s="77"/>
+      <c r="I59" s="77"/>
+      <c r="J59" s="77"/>
+      <c r="K59" s="77"/>
+      <c r="L59" s="77"/>
       <c r="N59" s="16"/>
       <c r="P59"/>
       <c r="Q59" s="16"/>
@@ -2007,15 +1982,15 @@
       <c r="C60" s="13"/>
       <c r="D60" s="17"/>
       <c r="E60" s="26"/>
-      <c r="F60" s="78" t="s">
+      <c r="F60" s="77" t="s">
         <v>14</v>
       </c>
-      <c r="G60" s="78"/>
-      <c r="H60" s="78"/>
-      <c r="I60" s="78"/>
-      <c r="J60" s="78"/>
-      <c r="K60" s="78"/>
-      <c r="L60" s="78"/>
+      <c r="G60" s="77"/>
+      <c r="H60" s="77"/>
+      <c r="I60" s="77"/>
+      <c r="J60" s="77"/>
+      <c r="K60" s="77"/>
+      <c r="L60" s="77"/>
       <c r="N60" s="16"/>
       <c r="P60" s="21"/>
       <c r="Q60" s="16"/>
@@ -2099,11 +2074,11 @@
         <v>10</v>
       </c>
       <c r="G65" s="13"/>
-      <c r="H65" s="74" t="s">
+      <c r="H65" s="73" t="s">
         <v>9</v>
       </c>
-      <c r="I65" s="74"/>
-      <c r="J65" s="74"/>
+      <c r="I65" s="73"/>
+      <c r="J65" s="73"/>
       <c r="N65" s="16"/>
       <c r="P65" s="19"/>
       <c r="Q65" s="16"/>
@@ -2117,11 +2092,11 @@
         <v>8</v>
       </c>
       <c r="G66" s="13"/>
-      <c r="H66" s="74" t="s">
+      <c r="H66" s="73" t="s">
         <v>7</v>
       </c>
-      <c r="I66" s="74"/>
-      <c r="J66" s="74"/>
+      <c r="I66" s="73"/>
+      <c r="J66" s="73"/>
       <c r="N66" s="16"/>
       <c r="P66" s="19"/>
       <c r="Q66" s="18"/>
@@ -2220,19 +2195,19 @@
       <c r="P73" s="6"/>
     </row>
     <row r="74" spans="2:17" ht="19">
-      <c r="B74" s="56" t="s">
+      <c r="B74" s="70" t="s">
         <v>0</v>
       </c>
-      <c r="C74" s="56"/>
-      <c r="D74" s="56"/>
-      <c r="E74" s="56"/>
-      <c r="F74" s="56"/>
-      <c r="G74" s="56"/>
-      <c r="H74" s="56"/>
-      <c r="I74" s="56"/>
-      <c r="J74" s="56"/>
-      <c r="K74" s="56"/>
-      <c r="L74" s="56"/>
+      <c r="C74" s="70"/>
+      <c r="D74" s="70"/>
+      <c r="E74" s="70"/>
+      <c r="F74" s="70"/>
+      <c r="G74" s="70"/>
+      <c r="H74" s="70"/>
+      <c r="I74" s="70"/>
+      <c r="J74" s="70"/>
+      <c r="K74" s="70"/>
+      <c r="L74" s="70"/>
     </row>
     <row r="75" spans="2:17">
       <c r="B75" s="4"/>
@@ -2951,6 +2926,114 @@
     </row>
   </sheetData>
   <mergeCells count="132">
+    <mergeCell ref="J13:L13"/>
+    <mergeCell ref="J14:L14"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="H2:L3"/>
+    <mergeCell ref="B5:E12"/>
+    <mergeCell ref="J5:L5"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="J8:L8"/>
+    <mergeCell ref="J9:L9"/>
+    <mergeCell ref="J10:L12"/>
+    <mergeCell ref="G29:I29"/>
+    <mergeCell ref="J29:J30"/>
+    <mergeCell ref="K29:K30"/>
+    <mergeCell ref="L29:L30"/>
+    <mergeCell ref="G30:I30"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="G20:I20"/>
+    <mergeCell ref="J27:J28"/>
+    <mergeCell ref="K27:K28"/>
+    <mergeCell ref="L27:L28"/>
+    <mergeCell ref="G21:I21"/>
+    <mergeCell ref="G22:I22"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="G23:I23"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="G27:I27"/>
+    <mergeCell ref="G28:I28"/>
+    <mergeCell ref="E29:E30"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="G31:I31"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="K31:K32"/>
+    <mergeCell ref="L31:L32"/>
+    <mergeCell ref="G32:I32"/>
+    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="F33:F34"/>
+    <mergeCell ref="G33:I33"/>
+    <mergeCell ref="J35:J36"/>
+    <mergeCell ref="K35:K36"/>
+    <mergeCell ref="L35:L36"/>
+    <mergeCell ref="G36:I36"/>
+    <mergeCell ref="E37:E38"/>
+    <mergeCell ref="F37:F38"/>
+    <mergeCell ref="G37:I37"/>
+    <mergeCell ref="J33:J34"/>
+    <mergeCell ref="K33:K34"/>
+    <mergeCell ref="L33:L34"/>
+    <mergeCell ref="G34:I34"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="H65:J65"/>
+    <mergeCell ref="H66:J66"/>
+    <mergeCell ref="B74:L74"/>
+    <mergeCell ref="E49:E50"/>
+    <mergeCell ref="F49:F50"/>
+    <mergeCell ref="G49:I49"/>
+    <mergeCell ref="G50:I50"/>
+    <mergeCell ref="F56:L56"/>
+    <mergeCell ref="F57:L57"/>
+    <mergeCell ref="F58:L58"/>
+    <mergeCell ref="F59:L59"/>
+    <mergeCell ref="F60:L60"/>
+    <mergeCell ref="L43:L44"/>
+    <mergeCell ref="G44:I44"/>
+    <mergeCell ref="F41:F42"/>
+    <mergeCell ref="G41:I41"/>
+    <mergeCell ref="J41:J42"/>
+    <mergeCell ref="K41:K42"/>
+    <mergeCell ref="L41:L42"/>
+    <mergeCell ref="G42:I42"/>
+    <mergeCell ref="E39:E40"/>
+    <mergeCell ref="F39:F40"/>
+    <mergeCell ref="K25:K26"/>
+    <mergeCell ref="L25:L26"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="K23:K24"/>
+    <mergeCell ref="E43:E44"/>
+    <mergeCell ref="F43:F44"/>
+    <mergeCell ref="G43:I43"/>
+    <mergeCell ref="J43:J44"/>
+    <mergeCell ref="K43:K44"/>
+    <mergeCell ref="G25:I25"/>
+    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="E41:E42"/>
+    <mergeCell ref="G39:I39"/>
+    <mergeCell ref="J39:J40"/>
+    <mergeCell ref="K39:K40"/>
+    <mergeCell ref="L39:L40"/>
+    <mergeCell ref="G40:I40"/>
+    <mergeCell ref="J37:J38"/>
+    <mergeCell ref="K37:K38"/>
+    <mergeCell ref="L37:L38"/>
+    <mergeCell ref="G38:I38"/>
+    <mergeCell ref="E35:E36"/>
+    <mergeCell ref="F35:F36"/>
+    <mergeCell ref="G35:I35"/>
     <mergeCell ref="F29:F30"/>
     <mergeCell ref="K17:K18"/>
     <mergeCell ref="L17:L18"/>
@@ -2975,114 +3058,6 @@
     <mergeCell ref="J19:J20"/>
     <mergeCell ref="L23:L24"/>
     <mergeCell ref="J25:J26"/>
-    <mergeCell ref="K25:K26"/>
-    <mergeCell ref="L25:L26"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="K23:K24"/>
-    <mergeCell ref="E43:E44"/>
-    <mergeCell ref="F43:F44"/>
-    <mergeCell ref="G43:I43"/>
-    <mergeCell ref="J43:J44"/>
-    <mergeCell ref="K43:K44"/>
-    <mergeCell ref="G25:I25"/>
-    <mergeCell ref="G26:I26"/>
-    <mergeCell ref="E41:E42"/>
-    <mergeCell ref="G39:I39"/>
-    <mergeCell ref="J39:J40"/>
-    <mergeCell ref="K39:K40"/>
-    <mergeCell ref="L39:L40"/>
-    <mergeCell ref="G40:I40"/>
-    <mergeCell ref="J37:J38"/>
-    <mergeCell ref="K37:K38"/>
-    <mergeCell ref="L37:L38"/>
-    <mergeCell ref="G38:I38"/>
-    <mergeCell ref="E35:E36"/>
-    <mergeCell ref="F35:F36"/>
-    <mergeCell ref="G35:I35"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="F21:F22"/>
-    <mergeCell ref="H65:J65"/>
-    <mergeCell ref="H66:J66"/>
-    <mergeCell ref="B74:L74"/>
-    <mergeCell ref="E49:E50"/>
-    <mergeCell ref="F49:F50"/>
-    <mergeCell ref="G49:I49"/>
-    <mergeCell ref="G50:I50"/>
-    <mergeCell ref="F56:L56"/>
-    <mergeCell ref="F57:L57"/>
-    <mergeCell ref="F58:L58"/>
-    <mergeCell ref="F59:L59"/>
-    <mergeCell ref="F60:L60"/>
-    <mergeCell ref="L43:L44"/>
-    <mergeCell ref="G44:I44"/>
-    <mergeCell ref="F41:F42"/>
-    <mergeCell ref="G41:I41"/>
-    <mergeCell ref="J41:J42"/>
-    <mergeCell ref="K41:K42"/>
-    <mergeCell ref="L41:L42"/>
-    <mergeCell ref="G42:I42"/>
-    <mergeCell ref="E39:E40"/>
-    <mergeCell ref="F39:F40"/>
-    <mergeCell ref="J35:J36"/>
-    <mergeCell ref="K35:K36"/>
-    <mergeCell ref="L35:L36"/>
-    <mergeCell ref="G36:I36"/>
-    <mergeCell ref="E37:E38"/>
-    <mergeCell ref="F37:F38"/>
-    <mergeCell ref="G37:I37"/>
-    <mergeCell ref="J33:J34"/>
-    <mergeCell ref="K33:K34"/>
-    <mergeCell ref="L33:L34"/>
-    <mergeCell ref="G34:I34"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="G31:I31"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="K31:K32"/>
-    <mergeCell ref="L31:L32"/>
-    <mergeCell ref="G32:I32"/>
-    <mergeCell ref="E33:E34"/>
-    <mergeCell ref="F33:F34"/>
-    <mergeCell ref="G33:I33"/>
-    <mergeCell ref="G29:I29"/>
-    <mergeCell ref="J29:J30"/>
-    <mergeCell ref="K29:K30"/>
-    <mergeCell ref="L29:L30"/>
-    <mergeCell ref="G30:I30"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="G20:I20"/>
-    <mergeCell ref="J27:J28"/>
-    <mergeCell ref="K27:K28"/>
-    <mergeCell ref="L27:L28"/>
-    <mergeCell ref="G21:I21"/>
-    <mergeCell ref="G22:I22"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="G23:I23"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="G27:I27"/>
-    <mergeCell ref="G28:I28"/>
-    <mergeCell ref="E29:E30"/>
-    <mergeCell ref="J13:L13"/>
-    <mergeCell ref="J14:L14"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="G17:I17"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="H2:L3"/>
-    <mergeCell ref="B5:E12"/>
-    <mergeCell ref="J5:L5"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="J7:L7"/>
-    <mergeCell ref="J8:L8"/>
-    <mergeCell ref="J9:L9"/>
-    <mergeCell ref="J10:L12"/>
   </mergeCells>
   <phoneticPr fontId="30" type="noConversion"/>
   <pageMargins left="0.75" right="0" top="0.75" bottom="0.25" header="0.3" footer="0"/>

</xml_diff>